<commit_message>
Shoulder-sparing chest drafts, device week start, dev-only prototype videos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Exercises" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercises'!$A$1:$L$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercises'!$A$1:$L$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="B18" s="7">
-        <f>COUNTA(Exercises!$A$2:$A$72)</f>
+        <f>COUNTA(Exercises!$A$2:$A$75)</f>
         <v/>
       </c>
     </row>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B19" s="7">
-        <f>COUNTIF(Exercises!$K$2:$K$72,"Approve")</f>
+        <f>COUNTIF(Exercises!$K$2:$K$75,"Approve")</f>
         <v/>
       </c>
     </row>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B20" s="7">
-        <f>COUNTIF(Exercises!$K$2:$K$72,"Fix")</f>
+        <f>COUNTIF(Exercises!$K$2:$K$75,"Fix")</f>
         <v/>
       </c>
     </row>
@@ -795,7 +795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1895,175 +1895,338 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>neutral_grip_floor_press</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Neutral-grip floor press</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Mid chest (Pectoralis major · sternal head): primary, 0.9
+Triceps (Triceps brachii): secondary, 0.6
+Front shoulders (Deltoid · front head): secondary, 0.2</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Dumbbells</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Standing</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Elbow / wrist</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Lie on the floor, palms facing each other; lower until your upper arms touch the floor, then press up.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Main work</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>neutral_grip_machine_chest_press</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Neutral-grip machine chest press</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Mid chest (Pectoralis major · sternal head): primary, 1.0
+Triceps (Triceps brachii): secondary, 0.5
+Front shoulders (Deltoid · front head): secondary, 0.3</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support, Seated</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Palms facing in, handles at mid-chest; press out without locking your elbows, stop before your hands pass your chest on the way back.</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Main work</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>short_range_incline_push_up</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Short-range incline push-up</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Mid chest (Pectoralis major · sternal head): primary, 0.8
+Lower chest (Pectoralis major · lower fibers): secondary, 0.4
+Triceps (Triceps brachii): secondary, 0.4
+Front shoulders (Deltoid · front head): secondary, 0.2</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Elbow / wrist</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Hands on a bench, body straight; lower only halfway, then push back up.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Main work</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t>dumbbell_shoulder_press</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Dumbbell shoulder press</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Front shoulders (Deltoid · front head): primary, 1.0
 Triceps (Triceps brachii): secondary, 0.5
 Traps (Trapezius): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Dumbbells</t>
         </is>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E24" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>Shoulder, Neck</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Press the dumbbells overhead without arching your back.</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K21" s="6" t="n"/>
-      <c r="L21" s="6" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>band_front_raise</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Band front raise</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Front shoulders (Deltoid · front head): primary, 0.9</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="E22" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="E25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>Shoulder</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>Raise straight arms to shoulder height and lower slowly.</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K22" s="6" t="n"/>
-      <c r="L22" s="6" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>band_face_pull</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Band face pull</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Rear shoulders (Deltoid · rear head): primary, 1.0
 Upper back (Rhomboids and middle trapezius): secondary, 0.6
 Traps (Trapezius): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="E23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="E26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>Pull the band toward your face, elbows high and out.</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K23" s="6" t="n"/>
-      <c r="L23" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>one_arm_dumbbell_row</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>One-arm dumbbell row</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Upper back (Rhomboids and middle trapezius): primary, 0.9
 Lats (Latissimus dorsi): primary, 0.8
@@ -2071,692 +2234,692 @@
 Rear shoulders (Deltoid · rear head): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Dumbbells, Bench</t>
         </is>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E27" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>Hand on the bench; pull the dumbbell to your hip.</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K24" s="6" t="n"/>
-      <c r="L24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>band_row</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Band row</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Upper back (Rhomboids and middle trapezius): primary, 1.0
 Lats (Latissimus dorsi): secondary, 0.5
 Biceps (Biceps brachii): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="E25" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="E28" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>Pull the band to your ribs, squeezing your shoulder blades.</t>
         </is>
       </c>
-      <c r="J25" s="5" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>lat_pulldown</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Lat pulldown</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Lats (Latissimus dorsi): primary, 1.0
 Biceps (Biceps brachii): secondary, 0.5
 Upper back (Rhomboids and middle trapezius): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>Cable</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="E29" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Shoulder</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>Pull the bar to your upper chest, chest up.</t>
         </is>
       </c>
-      <c r="J26" s="5" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="K29" s="6" t="n"/>
+      <c r="L29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>seated_cable_row</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Seated cable row</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Upper back (Rhomboids and middle trapezius): primary, 1.0
 Lats (Latissimus dorsi): secondary, 0.6
 Biceps (Biceps brachii): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>Cable</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="E30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>Sit tall and pull the handle to your belly.</t>
         </is>
       </c>
-      <c r="J27" s="5" t="inlineStr">
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="K30" s="6" t="n"/>
+      <c r="L30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>dumbbell_shrug</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Dumbbell shrug</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Traps (Trapezius): primary, 1.0
 Forearms (Wrist flexors and extensors): stabilizer, 0.3</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Dumbbells</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="E31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>Neck</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>Lift your shoulders toward your ears, pause, lower.</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>superman</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Superman</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Lower back (Erector spinae): primary, 1.0
 Glutes (Gluteus maximus and medius): secondary, 0.5</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E29" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="E32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>Lower back, Pregnant / postpartum, Recent surgery</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>Lying face down, lift arms and legs a little, then lower.</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr">
+      <c r="J32" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="K32" s="6" t="n"/>
+      <c r="L32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>bird_dog</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Bird dog</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Lower back (Erector spinae): primary, 0.8
 Glutes (Gluteus maximus and medius): secondary, 0.5
 Lower abs (Rectus abdominis · lower): stabilizer, 0.4</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="E33" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>Recent surgery</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr">
         <is>
           <t>On hands and knees, reach one arm and the opposite leg long.</t>
         </is>
       </c>
-      <c r="J30" s="5" t="inlineStr">
+      <c r="J33" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="K33" s="6" t="n"/>
+      <c r="L33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>dumbbell_curl</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Dumbbell curl</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Biceps (Biceps brachii): primary, 1.0
 Forearms (Wrist flexors and extensors): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>Dumbbells</t>
         </is>
       </c>
-      <c r="E31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="E34" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>Elbow / wrist</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="I34" s="5" t="inlineStr">
         <is>
           <t>Elbows by your sides; curl up and lower slowly.</t>
         </is>
       </c>
-      <c r="J31" s="5" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="6" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="K34" s="6" t="n"/>
+      <c r="L34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>band_curl</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Band curl</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Biceps (Biceps brachii): primary, 0.9
 Forearms (Wrist flexors and extensors): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="E32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="E35" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H32" s="5" t="inlineStr">
+      <c r="H35" s="5" t="inlineStr">
         <is>
           <t>Elbow / wrist</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>Stand on the band and curl your hands to your shoulders.</t>
         </is>
       </c>
-      <c r="J32" s="5" t="inlineStr">
+      <c r="J35" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="K35" s="6" t="n"/>
+      <c r="L35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>overhead_dumbbell_triceps_extension</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Overhead triceps extension</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Triceps (Triceps brachii): primary, 1.0</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Dumbbells</t>
         </is>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="E36" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>Shoulder, Elbow / wrist</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>Hold a dumbbell overhead; lower behind your head and extend.</t>
         </is>
       </c>
-      <c r="J33" s="5" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="6" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="K36" s="6" t="n"/>
+      <c r="L36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>bench_dip</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Bench dip</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Triceps (Triceps brachii): primary, 1.0
 Lower chest (Pectoralis major · lower fibers): secondary, 0.4
 Front shoulders (Deltoid · front head): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>Bench</t>
         </is>
       </c>
-      <c r="E34" s="5" t="n">
+      <c r="E37" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="H37" s="5" t="inlineStr">
         <is>
           <t>Shoulder, Elbow / wrist</t>
         </is>
       </c>
-      <c r="I34" s="5" t="inlineStr">
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>Hands on the bench behind you; bend your elbows and press up.</t>
         </is>
       </c>
-      <c r="J34" s="5" t="inlineStr">
+      <c r="J37" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="K37" s="6" t="n"/>
+      <c r="L37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>band_triceps_pushdown</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>Band triceps pushdown</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>Triceps (Triceps brachii): primary, 0.9</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="E35" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="E38" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>Elbow / wrist</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="I38" s="5" t="inlineStr">
         <is>
           <t>Elbows fixed at your sides; push the band down.</t>
         </is>
       </c>
-      <c r="J35" s="5" t="inlineStr">
+      <c r="J38" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K35" s="6" t="n"/>
-      <c r="L35" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="K38" s="6" t="n"/>
+      <c r="L38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>dumbbell_wrist_curl</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Dumbbell wrist curl</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>Forearms (Wrist flexors and extensors): primary, 1.0</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Dumbbells</t>
         </is>
       </c>
-      <c r="E36" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="E39" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H39" s="5" t="inlineStr">
         <is>
           <t>Elbow / wrist</t>
         </is>
       </c>
-      <c r="I36" s="5" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>Forearms on your thighs; curl the dumbbells with your wrists.</t>
         </is>
       </c>
-      <c r="J36" s="5" t="inlineStr">
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="K39" s="6" t="n"/>
+      <c r="L39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>plank</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Plank</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Upper abs (Rectus abdominis · upper): primary, 0.7
 Lower abs (Rectus abdominis · lower): primary, 0.7
@@ -2764,1172 +2927,1172 @@
 Front shoulders (Deltoid · front head): stabilizer, 0.3</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E37" s="5" t="n">
+      <c r="E40" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="H40" s="5" t="inlineStr">
         <is>
           <t>Shoulder, Recent surgery, High blood pressure</t>
         </is>
       </c>
-      <c r="I37" s="5" t="inlineStr">
+      <c r="I40" s="5" t="inlineStr">
         <is>
           <t>Elbows under shoulders, body in a straight line. Breathe.</t>
         </is>
       </c>
-      <c r="J37" s="5" t="inlineStr">
+      <c r="J40" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K37" s="6" t="n"/>
-      <c r="L37" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="K40" s="6" t="n"/>
+      <c r="L40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>dead_bug</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Dead bug</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>Lower abs (Rectus abdominis · lower): primary, 1.0
 Upper abs (Rectus abdominis · upper): secondary, 0.5</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E38" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="E41" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H38" s="5" t="inlineStr">
+      <c r="H41" s="5" t="inlineStr">
         <is>
           <t>Pregnant / postpartum, Recent surgery</t>
         </is>
       </c>
-      <c r="I38" s="5" t="inlineStr">
+      <c r="I41" s="5" t="inlineStr">
         <is>
           <t>On your back, lower the opposite arm and leg, low back down.</t>
         </is>
       </c>
-      <c r="J38" s="5" t="inlineStr">
+      <c r="J41" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K38" s="6" t="n"/>
-      <c r="L38" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="K41" s="6" t="n"/>
+      <c r="L41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>crunch</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>Crunch</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>Upper abs (Rectus abdominis · upper): primary, 1.0
 Lower abs (Rectus abdominis · lower): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E39" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="E42" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="H42" s="5" t="inlineStr">
         <is>
           <t>Neck, Pregnant / postpartum, Recent surgery, Osteoporosis</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="I42" s="5" t="inlineStr">
         <is>
           <t>Knees bent; curl your shoulders off the floor, then lower.</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
+      <c r="J42" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K39" s="6" t="n"/>
-      <c r="L39" s="6" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="K42" s="6" t="n"/>
+      <c r="L42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>reverse_crunch</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>Reverse crunch</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>Lower abs (Rectus abdominis · lower): primary, 1.0
 Upper abs (Rectus abdominis · upper): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E40" s="5" t="n">
+      <c r="E43" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H40" s="5" t="inlineStr">
+      <c r="H43" s="5" t="inlineStr">
         <is>
           <t>Lower back, Pregnant / postpartum, Recent surgery</t>
         </is>
       </c>
-      <c r="I40" s="5" t="inlineStr">
+      <c r="I43" s="5" t="inlineStr">
         <is>
           <t>On your back, curl your knees toward your chest.</t>
         </is>
       </c>
-      <c r="J40" s="5" t="inlineStr">
+      <c r="J43" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K40" s="6" t="n"/>
-      <c r="L40" s="6" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="K43" s="6" t="n"/>
+      <c r="L43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>side_plank</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>Side plank</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>Obliques (External and internal obliques): primary, 1.0
 Lower abs (Rectus abdominis · lower): secondary, 0.3
 Hips (Hip flexors): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E41" s="5" t="n">
+      <c r="E44" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="H44" s="5" t="inlineStr">
         <is>
           <t>Shoulder, Recent surgery</t>
         </is>
       </c>
-      <c r="I41" s="5" t="inlineStr">
+      <c r="I44" s="5" t="inlineStr">
         <is>
           <t>On one elbow, lift your hips into a straight line.</t>
         </is>
       </c>
-      <c r="J41" s="5" t="inlineStr">
+      <c r="J44" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K41" s="6" t="n"/>
-      <c r="L41" s="6" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="K44" s="6" t="n"/>
+      <c r="L44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>band_pallof_press</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Band Pallof press</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Obliques (External and internal obliques): primary, 1.0
 Lower abs (Rectus abdominis · lower): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="E42" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="E45" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
+      <c r="H45" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I42" s="5" t="inlineStr">
+      <c r="I45" s="5" t="inlineStr">
         <is>
           <t>Band at your side; press it straight out and resist the twist.</t>
         </is>
       </c>
-      <c r="J42" s="5" t="inlineStr">
+      <c r="J45" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K42" s="6" t="n"/>
-      <c r="L42" s="6" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="K45" s="6" t="n"/>
+      <c r="L45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>bodyweight_squat</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>Bodyweight squat</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 1.0
 Glutes (Gluteus maximus and medius): secondary, 0.7
 Inner thighs (Hip adductors): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E43" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="E46" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr">
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>Knee</t>
         </is>
       </c>
-      <c r="I43" s="5" t="inlineStr">
+      <c r="I46" s="5" t="inlineStr">
         <is>
           <t>Sit back and down, knees over toes, then stand.</t>
         </is>
       </c>
-      <c r="J43" s="5" t="inlineStr">
+      <c r="J46" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K43" s="6" t="n"/>
-      <c r="L43" s="6" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="K46" s="6" t="n"/>
+      <c r="L46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>goblet_squat</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>Goblet squat</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 1.0
 Glutes (Gluteus maximus and medius): secondary, 0.7
 Upper abs (Rectus abdominis · upper): stabilizer, 0.3</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Dumbbells</t>
         </is>
       </c>
-      <c r="E44" s="5" t="n">
+      <c r="E47" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H44" s="5" t="inlineStr">
+      <c r="H47" s="5" t="inlineStr">
         <is>
           <t>Knee, Lower back</t>
         </is>
       </c>
-      <c r="I44" s="5" t="inlineStr">
+      <c r="I47" s="5" t="inlineStr">
         <is>
           <t>Hold a dumbbell at your chest; squat down and stand tall.</t>
         </is>
       </c>
-      <c r="J44" s="5" t="inlineStr">
+      <c r="J47" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K44" s="6" t="n"/>
-      <c r="L44" s="6" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="K47" s="6" t="n"/>
+      <c r="L47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
         <is>
           <t>sit_to_stand</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>Sit to stand</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 0.9
 Glutes (Gluteus maximus and medius): secondary, 0.7</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E45" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="E48" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr">
+      <c r="H48" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I45" s="5" t="inlineStr">
+      <c r="I48" s="5" t="inlineStr">
         <is>
           <t>From a chair, stand up without using your hands, then sit slowly.</t>
         </is>
       </c>
-      <c r="J45" s="5" t="inlineStr">
+      <c r="J48" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K45" s="6" t="n"/>
-      <c r="L45" s="6" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="K48" s="6" t="n"/>
+      <c r="L48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>reverse_lunge</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Reverse lunge</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 0.8
 Glutes (Gluteus maximus and medius): primary, 0.8
 Inner thighs (Hip adductors): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E46" s="5" t="n">
+      <c r="E49" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H46" s="5" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>Knee, Hip, Ankle / foot, Fell in the last year</t>
         </is>
       </c>
-      <c r="I46" s="5" t="inlineStr">
+      <c r="I49" s="5" t="inlineStr">
         <is>
           <t>Step back and lower both knees, then return.</t>
         </is>
       </c>
-      <c r="J46" s="5" t="inlineStr">
+      <c r="J49" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K46" s="6" t="n"/>
-      <c r="L46" s="6" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="K49" s="6" t="n"/>
+      <c r="L49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>leg_press</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>Leg press</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 1.0
 Glutes (Gluteus maximus and medius): secondary, 0.6</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="E47" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="E50" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="G50" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr">
+      <c r="H50" s="5" t="inlineStr">
         <is>
           <t>Knee, Lower back</t>
         </is>
       </c>
-      <c r="I47" s="5" t="inlineStr">
+      <c r="I50" s="5" t="inlineStr">
         <is>
           <t>Feet hip-width; lower with control and press away.</t>
         </is>
       </c>
-      <c r="J47" s="5" t="inlineStr">
+      <c r="J50" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K47" s="6" t="n"/>
-      <c r="L47" s="6" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
+      <c r="K50" s="6" t="n"/>
+      <c r="L50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>glute_bridge</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Glute bridge</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Glutes (Gluteus maximus and medius): primary, 1.0
 Hamstrings (Hamstrings): secondary, 0.5
 Lower back (Erector spinae): stabilizer, 0.2</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E48" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="E51" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H48" s="5" t="inlineStr">
+      <c r="H51" s="5" t="inlineStr">
         <is>
           <t>Pregnant / postpartum</t>
         </is>
       </c>
-      <c r="I48" s="5" t="inlineStr">
+      <c r="I51" s="5" t="inlineStr">
         <is>
           <t>On your back, drive through your heels and lift your hips.</t>
         </is>
       </c>
-      <c r="J48" s="5" t="inlineStr">
+      <c r="J51" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K48" s="6" t="n"/>
-      <c r="L48" s="6" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
+      <c r="K51" s="6" t="n"/>
+      <c r="L51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>dumbbell_romanian_deadlift</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>Dumbbell Romanian deadlift</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Hamstrings (Hamstrings): primary, 1.0
 Glutes (Gluteus maximus and medius): primary, 0.8
 Lower back (Erector spinae): secondary, 0.5</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>Dumbbells</t>
         </is>
       </c>
-      <c r="E49" s="5" t="n">
+      <c r="E52" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F52" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G52" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr">
+      <c r="H52" s="5" t="inlineStr">
         <is>
           <t>Lower back, Recent surgery</t>
         </is>
       </c>
-      <c r="I49" s="5" t="inlineStr">
+      <c r="I52" s="5" t="inlineStr">
         <is>
           <t>Soft knees; hinge at the hips, dumbbells close to your legs.</t>
         </is>
       </c>
-      <c r="J49" s="5" t="inlineStr">
+      <c r="J52" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K49" s="6" t="n"/>
-      <c r="L49" s="6" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="K52" s="6" t="n"/>
+      <c r="L52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>lying_hamstring_curl_machine</t>
         </is>
       </c>
-      <c r="B50" s="5" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>Lying hamstring curl</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Hamstrings (Hamstrings): primary, 1.0
 Calves (Gastrocnemius and soleus): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>Machine</t>
         </is>
       </c>
-      <c r="E50" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="E53" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
         <is>
           <t>13+ (teens)</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="G53" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H50" s="5" t="inlineStr">
+      <c r="H53" s="5" t="inlineStr">
         <is>
           <t>Knee</t>
         </is>
       </c>
-      <c r="I50" s="5" t="inlineStr">
+      <c r="I53" s="5" t="inlineStr">
         <is>
           <t>Curl your heels toward your glutes and lower slowly.</t>
         </is>
       </c>
-      <c r="J50" s="5" t="inlineStr">
+      <c r="J53" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K50" s="6" t="n"/>
-      <c r="L50" s="6" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
+      <c r="K53" s="6" t="n"/>
+      <c r="L53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>standing_calf_raise</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Standing calf raise</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Calves (Gastrocnemius and soleus): primary, 1.0</t>
         </is>
       </c>
-      <c r="D51" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E51" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="E54" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H51" s="5" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>Ankle / foot</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr">
+      <c r="I54" s="5" t="inlineStr">
         <is>
           <t>Rise onto your toes, pause, lower slowly.</t>
         </is>
       </c>
-      <c r="J51" s="5" t="inlineStr">
+      <c r="J54" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K51" s="6" t="n"/>
-      <c r="L51" s="6" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="K54" s="6" t="n"/>
+      <c r="L54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>seated_knee_raise</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Seated knee raise</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Hips (Hip flexors): primary, 1.0
 Lower abs (Rectus abdominis · lower): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E52" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="E55" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>Hip</t>
         </is>
       </c>
-      <c r="I52" s="5" t="inlineStr">
+      <c r="I55" s="5" t="inlineStr">
         <is>
           <t>Sit tall and lift one knee toward your chest.</t>
         </is>
       </c>
-      <c r="J52" s="5" t="inlineStr">
+      <c r="J55" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K52" s="6" t="n"/>
-      <c r="L52" s="6" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+      <c r="K55" s="6" t="n"/>
+      <c r="L55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
         <is>
           <t>side_lying_adductor_raise</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>Side-lying inner thigh raise</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Inner thighs (Hip adductors): primary, 1.0</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E53" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="E56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H53" s="5" t="inlineStr">
+      <c r="H56" s="5" t="inlineStr">
         <is>
           <t>Hip</t>
         </is>
       </c>
-      <c r="I53" s="5" t="inlineStr">
+      <c r="I56" s="5" t="inlineStr">
         <is>
           <t>Lying on your side, lift the bottom leg a little.</t>
         </is>
       </c>
-      <c r="J53" s="5" t="inlineStr">
+      <c r="J56" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K53" s="6" t="n"/>
-      <c r="L53" s="6" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
+      <c r="K56" s="6" t="n"/>
+      <c r="L56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>wall_tibialis_raise</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>Wall tibialis raise</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Shins (Tibialis anterior): primary, 1.0</t>
         </is>
       </c>
-      <c r="D54" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E54" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
+      <c r="E57" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H54" s="5" t="inlineStr">
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>Ankle / foot</t>
         </is>
       </c>
-      <c r="I54" s="5" t="inlineStr">
+      <c r="I57" s="5" t="inlineStr">
         <is>
           <t>Back on a wall, lift your toes up and lower.</t>
         </is>
       </c>
-      <c r="J54" s="5" t="inlineStr">
+      <c r="J57" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K54" s="6" t="n"/>
-      <c r="L54" s="6" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="5" t="inlineStr">
+      <c r="K57" s="6" t="n"/>
+      <c r="L57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>band_terminal_knee_extension</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr">
         <is>
           <t>Band knee extension</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>Knees (Muscles around the knee): primary, 0.8
 Quads (Quadriceps): primary, 0.7</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>Bands</t>
         </is>
       </c>
-      <c r="E55" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="E58" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H55" s="5" t="inlineStr">
+      <c r="H58" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I55" s="5" t="inlineStr">
+      <c r="I58" s="5" t="inlineStr">
         <is>
           <t>Band behind your knee; straighten the knee against it.</t>
         </is>
       </c>
-      <c r="J55" s="5" t="inlineStr">
+      <c r="J58" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K55" s="6" t="n"/>
-      <c r="L55" s="6" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="K58" s="6" t="n"/>
+      <c r="L58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>step_up</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>Step-up</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 0.9
 Glutes (Gluteus maximus and medius): primary, 0.7</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>Bench</t>
         </is>
       </c>
-      <c r="E56" s="5" t="n">
+      <c r="E59" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H56" s="5" t="inlineStr">
+      <c r="H59" s="5" t="inlineStr">
         <is>
           <t>Knee, Ankle / foot, Fell in the last year</t>
         </is>
       </c>
-      <c r="I56" s="5" t="inlineStr">
+      <c r="I59" s="5" t="inlineStr">
         <is>
           <t>Step onto the bench, stand tall, step down with control.</t>
         </is>
       </c>
-      <c r="J56" s="5" t="inlineStr">
+      <c r="J59" s="5" t="inlineStr">
         <is>
           <t>Main work, Finisher: cardio</t>
         </is>
       </c>
-      <c r="K56" s="6" t="n"/>
-      <c r="L56" s="6" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="5" t="inlineStr">
+      <c r="K59" s="6" t="n"/>
+      <c r="L59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
         <is>
           <t>single_leg_balance</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>Single-leg balance</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Calves (Gastrocnemius and soleus): primary, 0.6
 Glutes (Gluteus maximus and medius): secondary, 0.5
 Shins (Tibialis anterior): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E57" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F57" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="E60" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H57" s="5" t="inlineStr">
+      <c r="H60" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I57" s="5" t="inlineStr">
+      <c r="I60" s="5" t="inlineStr">
         <is>
           <t>Stand on one leg; hold a support if you need it.</t>
         </is>
       </c>
-      <c r="J57" s="5" t="inlineStr">
+      <c r="J60" s="5" t="inlineStr">
         <is>
           <t>Main work, Finisher: mobility</t>
         </is>
       </c>
-      <c r="K57" s="6" t="n"/>
-      <c r="L57" s="6" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="K60" s="6" t="n"/>
+      <c r="L60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>mountain_climber</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>Mountain climber</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Lower abs (Rectus abdominis · lower): primary, 0.6
 Hips (Hip flexors): secondary, 0.5
 Front shoulders (Deltoid · front head): stabilizer, 0.4</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E58" s="5" t="n">
+      <c r="E61" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H58" s="5" t="inlineStr">
+      <c r="H61" s="5" t="inlineStr">
         <is>
           <t>Shoulder, Elbow / wrist, Heart condition, Pregnant / postpartum, Recent surgery, High blood pressure</t>
         </is>
       </c>
-      <c r="I58" s="5" t="inlineStr">
+      <c r="I61" s="5" t="inlineStr">
         <is>
           <t>In a plank, drive your knees in, one after the other.</t>
         </is>
       </c>
-      <c r="J58" s="5" t="inlineStr">
+      <c r="J61" s="5" t="inlineStr">
         <is>
           <t>Finisher: cardio</t>
         </is>
       </c>
-      <c r="K58" s="6" t="n"/>
-      <c r="L58" s="6" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="K61" s="6" t="n"/>
+      <c r="L61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
         <is>
           <t>doorway_chest_stretch</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>Doorway chest stretch</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Mid chest (Pectoralis major · sternal head): primary, 0.8
 Upper chest (Pectoralis major · clavicular head): secondary, 0.6
@@ -3937,735 +4100,735 @@
 Front shoulders (Deltoid · front head): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E59" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
+      <c r="E62" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H59" s="5" t="inlineStr">
+      <c r="H62" s="5" t="inlineStr">
         <is>
           <t>Shoulder</t>
         </is>
       </c>
-      <c r="I59" s="5" t="inlineStr">
+      <c r="I62" s="5" t="inlineStr">
         <is>
           <t>Forearm on a door frame; lean forward gently.</t>
         </is>
       </c>
-      <c r="J59" s="5" t="inlineStr">
+      <c r="J62" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch, Finisher: mobility</t>
         </is>
       </c>
-      <c r="K59" s="6" t="n"/>
-      <c r="L59" s="6" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+      <c r="K62" s="6" t="n"/>
+      <c r="L62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>cross_body_shoulder_stretch</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>Cross-body shoulder stretch</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Rear shoulders (Deltoid · rear head): primary, 0.8
 Front shoulders (Deltoid · front head): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E60" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
+      <c r="E63" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H60" s="5" t="inlineStr">
+      <c r="H63" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I60" s="5" t="inlineStr">
+      <c r="I63" s="5" t="inlineStr">
         <is>
           <t>Pull one arm across your chest with the other.</t>
         </is>
       </c>
-      <c r="J60" s="5" t="inlineStr">
+      <c r="J63" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K60" s="6" t="n"/>
-      <c r="L60" s="6" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
+      <c r="K63" s="6" t="n"/>
+      <c r="L63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
         <is>
           <t>overhead_triceps_stretch</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B64" s="5" t="inlineStr">
         <is>
           <t>Overhead triceps stretch</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C64" s="5" t="inlineStr">
         <is>
           <t>Triceps (Triceps brachii): primary, 0.8
 Lats (Latissimus dorsi): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E61" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="E64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H61" s="5" t="inlineStr">
+      <c r="H64" s="5" t="inlineStr">
         <is>
           <t>Shoulder</t>
         </is>
       </c>
-      <c r="I61" s="5" t="inlineStr">
+      <c r="I64" s="5" t="inlineStr">
         <is>
           <t>Hand behind your head; gently press the elbow.</t>
         </is>
       </c>
-      <c r="J61" s="5" t="inlineStr">
+      <c r="J64" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K61" s="6" t="n"/>
-      <c r="L61" s="6" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="K64" s="6" t="n"/>
+      <c r="L64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>standing_quad_stretch</t>
         </is>
       </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>Standing quad stretch</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 0.9
 Hips (Hip flexors): secondary, 0.4
 Knees (Muscles around the knee): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E62" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
+      <c r="E65" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H62" s="5" t="inlineStr">
+      <c r="H65" s="5" t="inlineStr">
         <is>
           <t>Knee</t>
         </is>
       </c>
-      <c r="I62" s="5" t="inlineStr">
+      <c r="I65" s="5" t="inlineStr">
         <is>
           <t>Hold a support; pull your heel toward your glute.</t>
         </is>
       </c>
-      <c r="J62" s="5" t="inlineStr">
+      <c r="J65" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K62" s="6" t="n"/>
-      <c r="L62" s="6" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="5" t="inlineStr">
+      <c r="K65" s="6" t="n"/>
+      <c r="L65" s="6" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
         <is>
           <t>seated_hamstring_stretch</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B66" s="5" t="inlineStr">
         <is>
           <t>Seated hamstring stretch</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C66" s="5" t="inlineStr">
         <is>
           <t>Hamstrings (Hamstrings): primary, 0.9
 Calves (Gastrocnemius and soleus): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="D66" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E63" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F63" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="inlineStr">
+      <c r="E66" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H63" s="5" t="inlineStr">
+      <c r="H66" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I63" s="5" t="inlineStr">
+      <c r="I66" s="5" t="inlineStr">
         <is>
           <t>Leg straight; lean forward from the hips.</t>
         </is>
       </c>
-      <c r="J63" s="5" t="inlineStr">
+      <c r="J66" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K63" s="6" t="n"/>
-      <c r="L63" s="6" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+      <c r="K66" s="6" t="n"/>
+      <c r="L66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>seated_figure_four_stretch</t>
         </is>
       </c>
-      <c r="B64" s="5" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>Seated figure-four stretch</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>Glutes (Gluteus maximus and medius): primary, 0.9
 Hips (Hip flexors): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E64" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
+      <c r="E67" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H64" s="5" t="inlineStr">
+      <c r="H67" s="5" t="inlineStr">
         <is>
           <t>Hip, Knee</t>
         </is>
       </c>
-      <c r="I64" s="5" t="inlineStr">
+      <c r="I67" s="5" t="inlineStr">
         <is>
           <t>Ankle over the other knee; lean forward gently.</t>
         </is>
       </c>
-      <c r="J64" s="5" t="inlineStr">
+      <c r="J67" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K64" s="6" t="n"/>
-      <c r="L64" s="6" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="K67" s="6" t="n"/>
+      <c r="L67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
         <is>
           <t>wall_calf_stretch</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>Wall calf stretch</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>Calves (Gastrocnemius and soleus): primary, 0.9
 Shins (Tibialis anterior): secondary, 0.3</t>
         </is>
       </c>
-      <c r="D65" s="5" t="inlineStr">
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E65" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="inlineStr">
+      <c r="E68" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H65" s="5" t="inlineStr">
+      <c r="H68" s="5" t="inlineStr">
         <is>
           <t>Ankle / foot</t>
         </is>
       </c>
-      <c r="I65" s="5" t="inlineStr">
+      <c r="I68" s="5" t="inlineStr">
         <is>
           <t>Hands on a wall, back leg straight, heel down.</t>
         </is>
       </c>
-      <c r="J65" s="5" t="inlineStr">
+      <c r="J68" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K65" s="6" t="n"/>
-      <c r="L65" s="6" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+      <c r="K68" s="6" t="n"/>
+      <c r="L68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>childs_pose</t>
         </is>
       </c>
-      <c r="B66" s="5" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>Child's pose</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>Lats (Latissimus dorsi): primary, 0.7
 Lower back (Erector spinae): primary, 0.6
 Upper back (Rhomboids and middle trapezius): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D66" s="5" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E66" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="inlineStr">
+      <c r="E69" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H66" s="5" t="inlineStr">
+      <c r="H69" s="5" t="inlineStr">
         <is>
           <t>Knee</t>
         </is>
       </c>
-      <c r="I66" s="5" t="inlineStr">
+      <c r="I69" s="5" t="inlineStr">
         <is>
           <t>Sit back on your heels and reach your arms forward.</t>
         </is>
       </c>
-      <c r="J66" s="5" t="inlineStr">
+      <c r="J69" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch, Finisher: mobility</t>
         </is>
       </c>
-      <c r="K66" s="6" t="n"/>
-      <c r="L66" s="6" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="5" t="inlineStr">
+      <c r="K69" s="6" t="n"/>
+      <c r="L69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t>kneeling_hip_flexor_stretch</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr">
+      <c r="B70" s="5" t="inlineStr">
         <is>
           <t>Kneeling hip flexor stretch</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>Hips (Hip flexors): primary, 0.9
 Quads (Quadriceps): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D67" s="5" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E67" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="inlineStr">
+      <c r="E70" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
         <is>
           <t>Standing</t>
         </is>
       </c>
-      <c r="H67" s="5" t="inlineStr">
+      <c r="H70" s="5" t="inlineStr">
         <is>
           <t>Knee</t>
         </is>
       </c>
-      <c r="I67" s="5" t="inlineStr">
+      <c r="I70" s="5" t="inlineStr">
         <is>
           <t>One knee down; shift your hips forward gently.</t>
         </is>
       </c>
-      <c r="J67" s="5" t="inlineStr">
+      <c r="J70" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch, Finisher: mobility</t>
         </is>
       </c>
-      <c r="K67" s="6" t="n"/>
-      <c r="L67" s="6" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+      <c r="K70" s="6" t="n"/>
+      <c r="L70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>upper_trap_stretch</t>
         </is>
       </c>
-      <c r="B68" s="5" t="inlineStr">
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>Upper trap stretch</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>Traps (Trapezius): primary, 0.8</t>
         </is>
       </c>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E68" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F68" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G68" s="5" t="inlineStr">
+      <c r="E71" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H68" s="5" t="inlineStr">
+      <c r="H71" s="5" t="inlineStr">
         <is>
           <t>Neck</t>
         </is>
       </c>
-      <c r="I68" s="5" t="inlineStr">
+      <c r="I71" s="5" t="inlineStr">
         <is>
           <t>Tilt your ear toward your shoulder; relax.</t>
         </is>
       </c>
-      <c r="J68" s="5" t="inlineStr">
+      <c r="J71" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K68" s="6" t="n"/>
-      <c r="L68" s="6" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+      <c r="K71" s="6" t="n"/>
+      <c r="L71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>standing_side_stretch</t>
         </is>
       </c>
-      <c r="B69" s="5" t="inlineStr">
+      <c r="B72" s="5" t="inlineStr">
         <is>
           <t>Side stretch</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
+      <c r="C72" s="5" t="inlineStr">
         <is>
           <t>Obliques (External and internal obliques): primary, 0.8
 Lats (Latissimus dorsi): secondary, 0.5</t>
         </is>
       </c>
-      <c r="D69" s="5" t="inlineStr">
+      <c r="D72" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E69" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G69" s="5" t="inlineStr">
+      <c r="E72" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H69" s="5" t="inlineStr">
+      <c r="H72" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I69" s="5" t="inlineStr">
+      <c r="I72" s="5" t="inlineStr">
         <is>
           <t>Reach one arm overhead and lean to the side.</t>
         </is>
       </c>
-      <c r="J69" s="5" t="inlineStr">
+      <c r="J72" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K69" s="6" t="n"/>
-      <c r="L69" s="6" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+      <c r="K72" s="6" t="n"/>
+      <c r="L72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t>hug_upper_back_stretch</t>
         </is>
       </c>
-      <c r="B70" s="5" t="inlineStr">
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>Upper back hug stretch</t>
         </is>
       </c>
-      <c r="C70" s="5" t="inlineStr">
+      <c r="C73" s="5" t="inlineStr">
         <is>
           <t>Upper back (Rhomboids and middle trapezius): primary, 0.8
 Rear shoulders (Deltoid · rear head): secondary, 0.4</t>
         </is>
       </c>
-      <c r="D70" s="5" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E70" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G70" s="5" t="inlineStr">
+      <c r="E73" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H70" s="5" t="inlineStr">
+      <c r="H73" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I70" s="5" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
         <is>
           <t>Hug yourself and round your upper back.</t>
         </is>
       </c>
-      <c r="J70" s="5" t="inlineStr">
+      <c r="J73" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K70" s="6" t="n"/>
-      <c r="L70" s="6" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
+      <c r="K73" s="6" t="n"/>
+      <c r="L73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t>biceps_wall_stretch</t>
         </is>
       </c>
-      <c r="B71" s="5" t="inlineStr">
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>Biceps wall stretch</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Biceps (Biceps brachii): primary, 0.8
 Forearms (Wrist flexors and extensors): secondary, 0.5</t>
         </is>
       </c>
-      <c r="D71" s="5" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E71" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="inlineStr">
+      <c r="E74" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H71" s="5" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
         <is>
           <t>Shoulder</t>
         </is>
       </c>
-      <c r="I71" s="5" t="inlineStr">
+      <c r="I74" s="5" t="inlineStr">
         <is>
           <t>Palm on a wall behind you; turn away slowly.</t>
         </is>
       </c>
-      <c r="J71" s="5" t="inlineStr">
+      <c r="J74" s="5" t="inlineStr">
         <is>
           <t>Cool-down: stretch</t>
         </is>
       </c>
-      <c r="K71" s="6" t="n"/>
-      <c r="L71" s="6" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
+      <c r="K74" s="6" t="n"/>
+      <c r="L74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>box_breathing</t>
         </is>
       </c>
-      <c r="B72" s="5" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Slow breathing</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>— (breathing, no muscle mapping)</t>
         </is>
       </c>
-      <c r="D72" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E72" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
+      <c r="E75" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
         <is>
           <t>Standing, With support, Seated</t>
         </is>
       </c>
-      <c r="H72" s="5" t="inlineStr">
+      <c r="H75" s="5" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I72" s="5" t="inlineStr">
+      <c r="I75" s="5" t="inlineStr">
         <is>
           <t>Breathe in for 4, hold 4, out for 4, hold 4.</t>
         </is>
       </c>
-      <c r="J72" s="5" t="inlineStr">
+      <c r="J75" s="5" t="inlineStr">
         <is>
           <t>Cool-down: breathing</t>
         </is>
       </c>
-      <c r="K72" s="6" t="n"/>
-      <c r="L72" s="6" t="n"/>
+      <c r="K75" s="6" t="n"/>
+      <c r="L75" s="6" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L72"/>
+  <autoFilter ref="A1:L75"/>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Approve or Fix." prompt="Approve, or Fix and explain in Comment." type="list">
+    <dataValidation sqref="K2:K75" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Approve or Fix." prompt="Approve, or Fix and explain in Comment." type="list">
       <formula1>"Approve,Fix"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Phase 7: progress, check-in, before/after, Repair and restrictions
- Progress tab with weekly sets chart, measurements (adults only) and links
- 4-week check-in: strength week 1 vs week 4, WHtR/BMI for adult and 60+ only
- Before/after photos on-device only, adult mode only
- Repair check (draft tests, dev builds only), guided test player, 6-week plan (Premium)
- My restrictions: impact, mark healed, manual add with side
- Family dashboard for the Family plan owner (workouts, minutes, streak)
- DB: checkins, repair_results, repair_plans with RLS; trigger refuses body
  fields for minors; session_kind 'repair'; revoke guard_managed_profiles
- Reviewer sheet gains a Repair tests tab; bundle check covers Repair drafts

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Exercises" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Repair tests" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercises'!$A$1:$L$75</definedName>
@@ -204,7 +205,7 @@
     <author>TapStrong</author>
   </authors>
   <commentList>
-    <comment ref="A24" authorId="0" shapeId="0">
+    <comment ref="A26" authorId="0" shapeId="0">
       <text>
         <t>Stored with each certified review (name + credential, e.g. NSCA-CSCS).</t>
       </text>
@@ -502,7 +503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -568,219 +569,237 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>4. Repair tests (tab "Repair tests"): are the protocol, the "good" target per age mode, the contraindications and the muscles each weak result sends to the 6-week plan right?</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>How to fill it in</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Only the two yellow columns on the "Exercises" tab: "Approve / Fix" (pick from the list) and "Comment". For "Fix", say what to change in the comment. Leave every other cell as it is.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Example (not part of the library):</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>ID (slug)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Exercise</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Muscles (role, emphasis 0–1)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Level (1–5)</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Minimum age</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Positions</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Contraindications</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Cues</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Used as</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Approve / Fix (Aprovado/Corrigir)</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Comment (Comentário)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>example_squat</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Example squat</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Quads (Quadriceps): primary, 1.0
 Glutes (Gluteus maximus and medius): secondary, 0.7</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Bodyweight</t>
         </is>
       </c>
-      <c r="E15" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>9+ (kids)</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="E16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>9+ (kids)</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Standing, With support</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>Knee</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Sit back and down, knees over toes, then stand.</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>Main work</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Fix</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>Add adductors as secondary, 0.3. Cue: keep heels down.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Progress (updates as you fill in the Exercises tab)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Exercises</t>
         </is>
       </c>
-      <c r="B18" s="7">
+      <c r="B19" s="7">
         <f>COUNTA(Exercises!$A$2:$A$75)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="B19" s="7">
+      <c r="B20" s="7">
         <f>COUNTIF(Exercises!$K$2:$K$75,"Approve")</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>To fix</t>
         </is>
       </c>
-      <c r="B20" s="7">
+      <c r="B21" s="7">
         <f>COUNTIF(Exercises!$K$2:$K$75,"Fix")</f>
         <v/>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Not reviewed yet</t>
         </is>
       </c>
-      <c r="B21" s="7">
-        <f>B18-B19-B20</f>
+      <c r="B22" s="7">
+        <f>B19-B20-B21</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Repair tests approved</t>
+        </is>
+      </c>
+      <c r="B23" s="7">
+        <f>COUNTIF('Repair tests'!$I$2:$I$6,"Approve")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Reviewer name, credential and date</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="9" t="n"/>
+    <row r="26">
+      <c r="A26" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Approve,Fix"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4834,4 +4853,307 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>How (shown to the user)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Result recorded</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Positions</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Contraindications</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>"Good" target by mode (kids / teens / adults / 60+)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Weak result → plan focus</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Approve / Fix (Aprovado/Corrigir)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Comment (Comentário)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>squat</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Sit-to-stand (30 s)</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Sit on a chair, arms crossed. Stand up fully and sit back down as many times as you can in 30 seconds. Count each full stand.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Reps in 30 s</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Knee, Recent surgery</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>15 reps / 15 reps / 15 reps / 12 reps</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Strengthen: Quads, Glutes</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>single_leg_balance</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Single-leg balance</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Stand on one leg, hands on hips, eyes open. Time how long you hold before the other foot touches down. Then the other leg.</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Hold time per side, seconds (max 60)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Ankle / foot, Recent surgery</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>20 s / 30 s / 30 s / 10 s</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Balance: Hips, Glutes</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>glute_bridge_hold</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Glute bridge hold</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Lie on your back, knees bent, feet flat. Lift your hips into a straight line from knees to shoulders and hold.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Hold time, seconds (max 60)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Standing</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Lower back, Recent surgery</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>20 s / 30 s / 30 s / 20 s</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Strengthen: Glutes, Hamstrings</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>front_plank</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Front plank</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Forearms and toes on the floor, body straight from head to heels. Hold without letting the hips sag.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Hold time, seconds (max 120)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Standing</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder, Lower back, Pregnant / postpartum, Recent surgery</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>20 s / 30 s / 45 s / 30 s</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Strengthen: Upper abs, Lower abs, Obliques</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>shoulder_reach</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Overhead shoulder reach</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Stand with your back against a wall. Raise one straight arm overhead. Can the back of your hand touch the wall without arching your back? Then the other arm.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Reached / limited, per side</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support, Seated</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder, Recent surgery</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Both sides reached</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Mobility: Front shoulders, Upper back</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="I2:I6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Approve,Fix"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add rotator cuff muscle; red light when the morning score is over 5
- rotatorCuff in the muscles table (no body-map hotspot), en/es/pt-BR
  labels; shoulder recovery focus and draft rehab exercise mappings use it
- Traffic light: next-morning score over 5 is red, as well as 2+ points
  above the previous score
- Reviewer sheet regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -5768,8 +5768,8 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Rear shoulders (Deltoid · rear head): primary, 0.6
-Front shoulders (Deltoid · front head): secondary, 0.4</t>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Rear shoulders (Deltoid · rear head): secondary, 0.4</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
@@ -5831,7 +5831,7 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Front shoulders (Deltoid · front head): primary, 0.5
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
 Chest (Pectoralis major): secondary, 0.3</t>
         </is>
       </c>
@@ -5894,7 +5894,8 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Front shoulders (Deltoid · front head): primary, 0.6</t>
+          <t>Front shoulders (Deltoid · front head): primary, 0.6
+Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): secondary, 0.5</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
@@ -5956,7 +5957,8 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Front shoulders (Deltoid · front head): primary, 0.6</t>
+          <t>Front shoulders (Deltoid · front head): primary, 0.6
+Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): secondary, 0.4</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
@@ -6018,7 +6020,8 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Rear shoulders (Deltoid · rear head): primary, 0.6
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Rear shoulders (Deltoid · rear head): secondary, 0.4
 Upper back (Rhomboids and middle trapezius): secondary, 0.3</t>
         </is>
       </c>
@@ -7687,7 +7690,7 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Shoulder: Front shoulders, Rear shoulders; Elbow: Forearms; Wrist: Forearms; Neck: Traps, Upper back; Lower back: Abs, Glutes; Hip: Glutes, Hips; Knee: Quads; Ankle: Calves, Shins</t>
+          <t>Shoulder: Rotator cuff, Rear shoulders; Elbow: Forearms; Wrist: Forearms; Neck: Traps, Upper back; Lower back: Abs, Glutes; Hip: Glutes, Hips; Knee: Quads; Ankle: Calves, Shins</t>
         </is>
       </c>
       <c r="E44" s="6" t="n"/>
@@ -7711,7 +7714,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Shoulder: Rear shoulders, Upper back, Front shoulders; Elbow: Forearms, Biceps, Triceps; Wrist: Forearms; Neck: Upper back, Traps, Rear shoulders; Lower back: Glutes, Obliques, Lower back; Hip: Glutes, Hips, Inner thighs; Knee: Quads, Glutes, Hamstrings; Ankle: Calves, Shins</t>
+          <t>Shoulder: Rotator cuff, Rear shoulders, Upper back; Elbow: Forearms, Biceps, Triceps; Wrist: Forearms; Neck: Upper back, Traps, Rear shoulders; Lower back: Glutes, Obliques, Lower back; Hip: Glutes, Hips, Inner thighs; Knee: Quads, Glutes, Hamstrings; Ankle: Calves, Shins</t>
         </is>
       </c>
       <c r="E45" s="6" t="n"/>
@@ -7735,7 +7738,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Shoulder: Front shoulders, Upper back, Chest, Lats; Elbow: Biceps, Triceps, Forearms; Wrist: Forearms, Biceps; Neck: Upper back, Traps, Front shoulders; Lower back: Lower back, Glutes, Hamstrings; Hip: Glutes, Quads, Hamstrings; Knee: Quads, Glutes, Calves; Ankle: Calves, Shins, Quads</t>
+          <t>Shoulder: Front shoulders, Rotator cuff, Upper back, Chest; Elbow: Biceps, Triceps, Forearms; Wrist: Forearms, Biceps; Neck: Upper back, Traps, Front shoulders; Lower back: Lower back, Glutes, Hamstrings; Hip: Glutes, Quads, Hamstrings; Knee: Quads, Glutes, Calves; Ankle: Calves, Shins, Quads</t>
         </is>
       </c>
       <c r="E46" s="6" t="n"/>

</xml_diff>

<commit_message>
Phase 13 P1: swap safety and two-handed loads (QA R3-07, R3-09)
- Swaps dose with jointCare like generation, and the ramp-up follows a
  swapped-in lift only when the generator would allow it.
- Recovery phase 1 leaves out holds contraindicated for the area in
  workouts, recovery sessions and swaps; recovery workouts swap with rehab
  rules and no shorter range.
- 40 loaded moves that need both hands lose the with_support position
  (split squat, single-leg RDL, standing curls, cable woodchop, ...), with a
  library audit test.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -2421,7 +2421,7 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
@@ -12768,7 +12768,7 @@
       </c>
       <c r="G183" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H183" s="5" t="inlineStr">
@@ -12959,7 +12959,7 @@
       </c>
       <c r="G186" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H186" s="5" t="inlineStr">
@@ -13093,7 +13093,7 @@
       </c>
       <c r="G188" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H188" s="5" t="inlineStr">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="G194" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H194" s="5" t="inlineStr">
@@ -13956,7 +13956,7 @@
       </c>
       <c r="G201" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H201" s="5" t="inlineStr">
@@ -14149,7 +14149,7 @@
       </c>
       <c r="G204" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H204" s="5" t="inlineStr">
@@ -14536,7 +14536,7 @@
       </c>
       <c r="G210" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H210" s="5" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="G215" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H215" s="5" t="inlineStr">
@@ -15060,7 +15060,7 @@
       </c>
       <c r="G218" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H218" s="5" t="inlineStr">
@@ -15582,7 +15582,7 @@
       </c>
       <c r="G226" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H226" s="5" t="inlineStr">
@@ -15648,7 +15648,7 @@
       </c>
       <c r="G227" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H227" s="5" t="inlineStr">
@@ -15781,7 +15781,7 @@
       </c>
       <c r="G229" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H229" s="5" t="inlineStr">
@@ -15849,7 +15849,7 @@
       </c>
       <c r="G230" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H230" s="5" t="inlineStr">
@@ -16044,7 +16044,7 @@
       </c>
       <c r="G233" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H233" s="5" t="inlineStr">
@@ -16173,7 +16173,7 @@
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H235" s="5" t="inlineStr">
@@ -16707,7 +16707,7 @@
       </c>
       <c r="G243" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H243" s="5" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="G245" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H245" s="5" t="inlineStr">
@@ -17029,7 +17029,7 @@
       </c>
       <c r="G248" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H248" s="5" t="inlineStr">
@@ -17092,7 +17092,7 @@
       </c>
       <c r="G249" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H249" s="5" t="inlineStr">
@@ -17155,7 +17155,7 @@
       </c>
       <c r="G250" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H250" s="5" t="inlineStr">
@@ -17353,7 +17353,7 @@
       </c>
       <c r="G253" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H253" s="5" t="inlineStr">
@@ -21082,7 +21082,7 @@
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H311" s="5" t="inlineStr">
@@ -21148,7 +21148,7 @@
       </c>
       <c r="G312" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H312" s="5" t="inlineStr">
@@ -21348,7 +21348,7 @@
       </c>
       <c r="G315" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H315" s="5" t="inlineStr">
@@ -22122,7 +22122,7 @@
       </c>
       <c r="G327" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H327" s="5" t="inlineStr">
@@ -22443,7 +22443,7 @@
       </c>
       <c r="G332" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H332" s="5" t="inlineStr">
@@ -28371,7 +28371,7 @@
       </c>
       <c r="G423" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H423" s="5" t="inlineStr">
@@ -28828,7 +28828,7 @@
       </c>
       <c r="G430" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support, Seated</t>
+          <t>Standing, Seated</t>
         </is>
       </c>
       <c r="H430" s="5" t="inlineStr">
@@ -44346,7 +44346,7 @@
       </c>
       <c r="G673" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H673" s="5" t="inlineStr">
@@ -44917,7 +44917,7 @@
       </c>
       <c r="G682" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H682" s="5" t="inlineStr">
@@ -44984,7 +44984,7 @@
       </c>
       <c r="G683" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H683" s="5" t="inlineStr">
@@ -47174,7 +47174,7 @@
       </c>
       <c r="G717" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H717" s="5" t="inlineStr">
@@ -47497,7 +47497,7 @@
       </c>
       <c r="G722" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H722" s="5" t="inlineStr">
@@ -47564,7 +47564,7 @@
       </c>
       <c r="G723" s="5" t="inlineStr">
         <is>
-          <t>Standing, With support</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H723" s="5" t="inlineStr">
@@ -48071,7 +48071,7 @@
       </c>
       <c r="G731" s="5" t="inlineStr">
         <is>
-          <t>With support, Standing</t>
+          <t>Standing</t>
         </is>
       </c>
       <c r="H731" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Phase 14 C: detailed equipment list, presets, saved places, exact filtering
- About 60 equipment items in groups (benches and racks, free weights,
  cables, machines by body part, bands and accessories, cardio), each with
  a switch under Settings > Equipment.
- Presets: Full gym, Small gym, Home gym, Bodyweight only, Hotel. Saved
  places (e.g. Gym and Home) with their own lists, switchable from a
  planned workout's header (the workout is rebuilt for that place).
- Seed: every exercise now lists the exact items it needs (machines and
  cables mapped one by one); the generator, swap sheet and library filter
  by the person's exact list. Old coarse answers and coach replies are
  read as items.
- Onboarding asks for a preset; the detailed list is optional.
- Coverage test: every preset keeps 5+ main options per muscle x position
  (no exemptions needed).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -1228,7 +1228,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Exercise bike</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Flat bench</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Chest press machine</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Chest press machine</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Adjustable bench</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
@@ -2742,7 +2742,7 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Lat pulldown</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Seated row (cable)</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Flat bench</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Leg press</t>
         </is>
       </c>
       <c r="E50" s="5" t="n">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Leg curl machine</t>
         </is>
       </c>
       <c r="E53" s="5" t="n">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E58" s="5" t="n">
@@ -4682,7 +4682,7 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Flat bench</t>
         </is>
       </c>
       <c r="E59" s="5" t="n">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E80" s="5" t="n">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="D130" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E130" s="5" t="n">
@@ -9351,7 +9351,7 @@
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E131" s="5" t="n">
@@ -9417,7 +9417,7 @@
       </c>
       <c r="D132" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E132" s="5" t="n">
@@ -9484,7 +9484,7 @@
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E133" s="5" t="n">
@@ -9551,7 +9551,7 @@
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E134" s="5" t="n">
@@ -9618,7 +9618,7 @@
       </c>
       <c r="D135" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E135" s="5" t="n">
@@ -9684,7 +9684,7 @@
       </c>
       <c r="D136" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E136" s="5" t="n">
@@ -9749,7 +9749,7 @@
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E137" s="5" t="n">
@@ -9814,7 +9814,7 @@
       </c>
       <c r="D138" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E138" s="5" t="n">
@@ -9880,7 +9880,7 @@
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E139" s="5" t="n">
@@ -9945,7 +9945,7 @@
       </c>
       <c r="D140" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E140" s="5" t="n">
@@ -10009,7 +10009,7 @@
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E141" s="5" t="n">
@@ -10073,7 +10073,7 @@
       </c>
       <c r="D142" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E142" s="5" t="n">
@@ -10138,7 +10138,7 @@
       </c>
       <c r="D143" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E143" s="5" t="n">
@@ -10203,7 +10203,7 @@
       </c>
       <c r="D144" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E144" s="5" t="n">
@@ -10267,7 +10267,7 @@
       </c>
       <c r="D145" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E145" s="5" t="n">
@@ -10331,7 +10331,7 @@
       </c>
       <c r="D146" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E146" s="5" t="n">
@@ -10396,7 +10396,7 @@
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E147" s="5" t="n">
@@ -10465,7 +10465,7 @@
       </c>
       <c r="D148" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E148" s="5" t="n">
@@ -10532,7 +10532,7 @@
       </c>
       <c r="D149" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E149" s="5" t="n">
@@ -10598,7 +10598,7 @@
       </c>
       <c r="D150" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E150" s="5" t="n">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="D151" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E151" s="5" t="n">
@@ -10729,7 +10729,7 @@
       </c>
       <c r="D152" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E152" s="5" t="n">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="D153" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E153" s="5" t="n">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="D154" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E154" s="5" t="n">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="D155" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E155" s="5" t="n">
@@ -10991,7 +10991,7 @@
       </c>
       <c r="D156" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E156" s="5" t="n">
@@ -11058,7 +11058,7 @@
       </c>
       <c r="D157" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E157" s="5" t="n">
@@ -11126,7 +11126,7 @@
       </c>
       <c r="D158" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E158" s="5" t="n">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="D159" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E159" s="5" t="n">
@@ -11260,7 +11260,7 @@
       </c>
       <c r="D160" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E160" s="5" t="n">
@@ -11325,7 +11325,7 @@
       </c>
       <c r="D161" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E161" s="5" t="n">
@@ -11389,7 +11389,7 @@
       </c>
       <c r="D162" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E162" s="5" t="n">
@@ -11453,7 +11453,7 @@
       </c>
       <c r="D163" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E163" s="5" t="n">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="D164" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E164" s="5" t="n">
@@ -11582,7 +11582,7 @@
       </c>
       <c r="D165" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E165" s="5" t="n">
@@ -11648,7 +11648,7 @@
       </c>
       <c r="D166" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E166" s="5" t="n">
@@ -11713,7 +11713,7 @@
       </c>
       <c r="D167" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E167" s="5" t="n">
@@ -11776,7 +11776,7 @@
       </c>
       <c r="D168" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E168" s="5" t="n">
@@ -11839,7 +11839,7 @@
       </c>
       <c r="D169" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E169" s="5" t="n">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="D170" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E170" s="5" t="n">
@@ -11966,7 +11966,7 @@
       </c>
       <c r="D171" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E171" s="5" t="n">
@@ -12031,7 +12031,7 @@
       </c>
       <c r="D172" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E172" s="5" t="n">
@@ -12098,7 +12098,7 @@
       </c>
       <c r="D173" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E173" s="5" t="n">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="D174" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E174" s="5" t="n">
@@ -12230,7 +12230,7 @@
       </c>
       <c r="D175" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E175" s="5" t="n">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="D176" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E176" s="5" t="n">
@@ -12625,7 +12625,7 @@
       </c>
       <c r="D181" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E181" s="5" t="n">
@@ -12691,7 +12691,7 @@
       </c>
       <c r="D182" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E182" s="5" t="n">
@@ -13216,7 +13216,7 @@
       </c>
       <c r="D190" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E190" s="5" t="n">
@@ -13412,7 +13412,7 @@
       </c>
       <c r="D193" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E193" s="5" t="n">
@@ -13610,7 +13610,7 @@
       </c>
       <c r="D196" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E196" s="5" t="n">
@@ -13676,7 +13676,7 @@
       </c>
       <c r="D197" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E197" s="5" t="n">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="D203" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Adjustable bench</t>
         </is>
       </c>
       <c r="E203" s="5" t="n">
@@ -14202,7 +14202,7 @@
       </c>
       <c r="D205" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E205" s="5" t="n">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="D207" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E207" s="5" t="n">
@@ -14654,7 +14654,7 @@
       </c>
       <c r="D212" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Chest press machine</t>
         </is>
       </c>
       <c r="E212" s="5" t="n">
@@ -14721,7 +14721,7 @@
       </c>
       <c r="D213" s="5" t="inlineStr">
         <is>
-          <t>Barbell, Bench</t>
+          <t>Barbell, Adjustable bench</t>
         </is>
       </c>
       <c r="E213" s="5" t="n">
@@ -14787,7 +14787,7 @@
       </c>
       <c r="D214" s="5" t="inlineStr">
         <is>
-          <t>Cable, Bench</t>
+          <t>Cable station, Adjustable bench</t>
         </is>
       </c>
       <c r="E214" s="5" t="n">
@@ -14853,7 +14853,7 @@
       </c>
       <c r="D215" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E215" s="5" t="n">
@@ -14920,7 +14920,7 @@
       </c>
       <c r="D216" s="5" t="inlineStr">
         <is>
-          <t>Barbell, Bench</t>
+          <t>Barbell, Flat bench</t>
         </is>
       </c>
       <c r="E216" s="5" t="n">
@@ -14985,7 +14985,7 @@
       </c>
       <c r="D217" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Pec deck</t>
         </is>
       </c>
       <c r="E217" s="5" t="n">
@@ -15049,7 +15049,7 @@
       </c>
       <c r="D218" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E218" s="5" t="n">
@@ -15114,7 +15114,7 @@
       </c>
       <c r="D219" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Assisted pull-up / dip machine</t>
         </is>
       </c>
       <c r="E219" s="5" t="n">
@@ -15182,7 +15182,7 @@
       </c>
       <c r="D220" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Dip station</t>
         </is>
       </c>
       <c r="E220" s="5" t="n">
@@ -15248,7 +15248,7 @@
       </c>
       <c r="D221" s="5" t="inlineStr">
         <is>
-          <t>Barbell, Bench</t>
+          <t>Barbell, Adjustable bench</t>
         </is>
       </c>
       <c r="E221" s="5" t="n">
@@ -15313,7 +15313,7 @@
       </c>
       <c r="D222" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E222" s="5" t="n">
@@ -15378,7 +15378,7 @@
       </c>
       <c r="D223" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Shoulder press machine</t>
         </is>
       </c>
       <c r="E223" s="5" t="n">
@@ -15445,7 +15445,7 @@
       </c>
       <c r="D224" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E224" s="5" t="n">
@@ -15509,7 +15509,7 @@
       </c>
       <c r="D225" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Lateral raise machine</t>
         </is>
       </c>
       <c r="E225" s="5" t="n">
@@ -15572,7 +15572,7 @@
       </c>
       <c r="D226" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E226" s="5" t="n">
@@ -15638,7 +15638,7 @@
       </c>
       <c r="D227" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E227" s="5" t="n">
@@ -15705,7 +15705,7 @@
       </c>
       <c r="D228" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Pec deck</t>
         </is>
       </c>
       <c r="E228" s="5" t="n">
@@ -15771,7 +15771,7 @@
       </c>
       <c r="D229" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E229" s="5" t="n">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="D230" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E230" s="5" t="n">
@@ -15903,7 +15903,7 @@
       </c>
       <c r="D231" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E231" s="5" t="n">
@@ -15969,7 +15969,7 @@
       </c>
       <c r="D232" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Seated row (cable)</t>
         </is>
       </c>
       <c r="E232" s="5" t="n">
@@ -16034,7 +16034,7 @@
       </c>
       <c r="D233" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E233" s="5" t="n">
@@ -16163,7 +16163,7 @@
       </c>
       <c r="D235" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E235" s="5" t="n">
@@ -16229,7 +16229,7 @@
       </c>
       <c r="D236" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Row machine</t>
         </is>
       </c>
       <c r="E236" s="5" t="n">
@@ -16364,7 +16364,7 @@
       </c>
       <c r="D238" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E238" s="5" t="n">
@@ -16430,7 +16430,7 @@
       </c>
       <c r="D239" s="5" t="inlineStr">
         <is>
-          <t>Barbell</t>
+          <t>Barbell, Squat rack</t>
         </is>
       </c>
       <c r="E239" s="5" t="n">
@@ -16630,7 +16630,7 @@
       </c>
       <c r="D242" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Assisted pull-up / dip machine</t>
         </is>
       </c>
       <c r="E242" s="5" t="n">
@@ -16698,7 +16698,7 @@
       </c>
       <c r="D243" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E243" s="5" t="n">
@@ -16763,7 +16763,7 @@
       </c>
       <c r="D244" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E244" s="5" t="n">
@@ -16829,7 +16829,7 @@
       </c>
       <c r="D245" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E245" s="5" t="n">
@@ -16956,7 +16956,7 @@
       </c>
       <c r="D247" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Preacher curl machine</t>
         </is>
       </c>
       <c r="E247" s="5" t="n">
@@ -17020,7 +17020,7 @@
       </c>
       <c r="D248" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E248" s="5" t="n">
@@ -17083,7 +17083,7 @@
       </c>
       <c r="D249" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E249" s="5" t="n">
@@ -17146,7 +17146,7 @@
       </c>
       <c r="D250" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E250" s="5" t="n">
@@ -17213,7 +17213,7 @@
       </c>
       <c r="D251" s="5" t="inlineStr">
         <is>
-          <t>Barbell, Bench</t>
+          <t>Barbell, Flat bench</t>
         </is>
       </c>
       <c r="E251" s="5" t="n">
@@ -17277,7 +17277,7 @@
       </c>
       <c r="D252" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E252" s="5" t="n">
@@ -17344,7 +17344,7 @@
       </c>
       <c r="D253" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E253" s="5" t="n">
@@ -17473,7 +17473,7 @@
       </c>
       <c r="D255" s="5" t="inlineStr">
         <is>
-          <t>Barbell, Bench</t>
+          <t>Barbell, Flat bench</t>
         </is>
       </c>
       <c r="E255" s="5" t="n">
@@ -20113,7 +20113,7 @@
       </c>
       <c r="D296" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E296" s="5" t="n">
@@ -20176,7 +20176,7 @@
       </c>
       <c r="D297" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E297" s="5" t="n">
@@ -20240,7 +20240,7 @@
       </c>
       <c r="D298" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E298" s="5" t="n">
@@ -20303,7 +20303,7 @@
       </c>
       <c r="D299" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E299" s="5" t="n">
@@ -20366,7 +20366,7 @@
       </c>
       <c r="D300" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E300" s="5" t="n">
@@ -20428,7 +20428,7 @@
       </c>
       <c r="D301" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E301" s="5" t="n">
@@ -20490,7 +20490,7 @@
       </c>
       <c r="D302" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E302" s="5" t="n">
@@ -20554,7 +20554,7 @@
       </c>
       <c r="D303" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E303" s="5" t="n">
@@ -20619,7 +20619,7 @@
       </c>
       <c r="D304" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E304" s="5" t="n">
@@ -20684,7 +20684,7 @@
       </c>
       <c r="D305" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E305" s="5" t="n">
@@ -20749,7 +20749,7 @@
       </c>
       <c r="D306" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E306" s="5" t="n">
@@ -20813,7 +20813,7 @@
       </c>
       <c r="D307" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E307" s="5" t="n">
@@ -20880,7 +20880,7 @@
       </c>
       <c r="D308" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E308" s="5" t="n">
@@ -20945,7 +20945,7 @@
       </c>
       <c r="D309" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E309" s="5" t="n">
@@ -21008,7 +21008,7 @@
       </c>
       <c r="D310" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E310" s="5" t="n">
@@ -21139,7 +21139,7 @@
       </c>
       <c r="D312" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E312" s="5" t="n">
@@ -21206,7 +21206,7 @@
       </c>
       <c r="D313" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E313" s="5" t="n">
@@ -21599,7 +21599,7 @@
       </c>
       <c r="D319" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Leg extension machine</t>
         </is>
       </c>
       <c r="E319" s="5" t="n">
@@ -21662,7 +21662,7 @@
       </c>
       <c r="D320" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Leg curl machine</t>
         </is>
       </c>
       <c r="E320" s="5" t="n">
@@ -21725,7 +21725,7 @@
       </c>
       <c r="D321" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Hip abductor / adductor</t>
         </is>
       </c>
       <c r="E321" s="5" t="n">
@@ -21787,7 +21787,7 @@
       </c>
       <c r="D322" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Hip abductor / adductor</t>
         </is>
       </c>
       <c r="E322" s="5" t="n">
@@ -21851,7 +21851,7 @@
       </c>
       <c r="D323" s="5" t="inlineStr">
         <is>
-          <t>Barbell</t>
+          <t>Barbell, Squat rack</t>
         </is>
       </c>
       <c r="E323" s="5" t="n">
@@ -21919,7 +21919,7 @@
       </c>
       <c r="D324" s="5" t="inlineStr">
         <is>
-          <t>Barbell, Bench</t>
+          <t>Barbell, Flat bench</t>
         </is>
       </c>
       <c r="E324" s="5" t="n">
@@ -21984,7 +21984,7 @@
       </c>
       <c r="D325" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E325" s="5" t="n">
@@ -22048,7 +22048,7 @@
       </c>
       <c r="D326" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Calf raise machine</t>
         </is>
       </c>
       <c r="E326" s="5" t="n">
@@ -22113,7 +22113,7 @@
       </c>
       <c r="D327" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E327" s="5" t="n">
@@ -22178,7 +22178,7 @@
       </c>
       <c r="D328" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E328" s="5" t="n">
@@ -22244,7 +22244,7 @@
       </c>
       <c r="D329" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Back extension bench</t>
         </is>
       </c>
       <c r="E329" s="5" t="n">
@@ -22308,7 +22308,7 @@
       </c>
       <c r="D330" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E330" s="5" t="n">
@@ -22371,7 +22371,7 @@
       </c>
       <c r="D331" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Ab crunch machine</t>
         </is>
       </c>
       <c r="E331" s="5" t="n">
@@ -22434,7 +22434,7 @@
       </c>
       <c r="D332" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E332" s="5" t="n">
@@ -28547,7 +28547,7 @@
       </c>
       <c r="D426" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E426" s="5" t="n">
@@ -28876,7 +28876,7 @@
       </c>
       <c r="D431" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E431" s="5" t="n">
@@ -28941,7 +28941,7 @@
       </c>
       <c r="D432" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E432" s="5" t="n">
@@ -29459,7 +29459,7 @@
       </c>
       <c r="D440" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E440" s="5" t="n">
@@ -29523,7 +29523,7 @@
       </c>
       <c r="D441" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E441" s="5" t="n">
@@ -30024,7 +30024,7 @@
       </c>
       <c r="D449" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E449" s="5" t="n">
@@ -31177,7 +31177,7 @@
       </c>
       <c r="D467" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E467" s="5" t="n">
@@ -31819,7 +31819,7 @@
       </c>
       <c r="D477" s="5" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Flat bench</t>
         </is>
       </c>
       <c r="E477" s="5" t="n">
@@ -32074,7 +32074,7 @@
       </c>
       <c r="D481" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E481" s="5" t="n">
@@ -32202,7 +32202,7 @@
       </c>
       <c r="D483" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E483" s="5" t="n">
@@ -32267,7 +32267,7 @@
       </c>
       <c r="D484" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E484" s="5" t="n">
@@ -32526,7 +32526,7 @@
       </c>
       <c r="D488" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E488" s="5" t="n">
@@ -32656,7 +32656,7 @@
       </c>
       <c r="D490" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E490" s="5" t="n">
@@ -33348,7 +33348,7 @@
       </c>
       <c r="D501" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E501" s="5" t="n">
@@ -33410,7 +33410,7 @@
       </c>
       <c r="D502" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E502" s="5" t="n">
@@ -33974,7 +33974,7 @@
       </c>
       <c r="D511" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Exercise bike</t>
         </is>
       </c>
       <c r="E511" s="5" t="n">
@@ -34687,7 +34687,7 @@
       </c>
       <c r="D522" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Rowing machine</t>
         </is>
       </c>
       <c r="E522" s="5" t="n">
@@ -34754,7 +34754,7 @@
       </c>
       <c r="D523" s="5" t="inlineStr">
         <is>
-          <t>Machine</t>
+          <t>Exercise bike</t>
         </is>
       </c>
       <c r="E523" s="5" t="n">
@@ -37701,7 +37701,7 @@
       </c>
       <c r="D569" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E569" s="5" t="n">
@@ -37768,7 +37768,7 @@
       </c>
       <c r="D570" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E570" s="5" t="n">
@@ -40504,7 +40504,7 @@
       </c>
       <c r="D613" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E613" s="5" t="n">
@@ -40567,7 +40567,7 @@
       </c>
       <c r="D614" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Mini bands</t>
         </is>
       </c>
       <c r="E614" s="5" t="n">
@@ -40945,7 +40945,7 @@
       </c>
       <c r="D620" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E620" s="5" t="n">
@@ -41007,7 +41007,7 @@
       </c>
       <c r="D621" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E621" s="5" t="n">
@@ -44530,7 +44530,7 @@
       </c>
       <c r="D676" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E676" s="5" t="n">
@@ -44724,7 +44724,7 @@
       </c>
       <c r="D679" s="5" t="inlineStr">
         <is>
-          <t>Kettlebell</t>
+          <t>Kettlebells</t>
         </is>
       </c>
       <c r="E679" s="5" t="n">
@@ -45231,7 +45231,7 @@
       </c>
       <c r="D687" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E687" s="5" t="n">
@@ -45295,7 +45295,7 @@
       </c>
       <c r="D688" s="5" t="inlineStr">
         <is>
-          <t>Kettlebell, Bench</t>
+          <t>Kettlebells, Flat bench</t>
         </is>
       </c>
       <c r="E688" s="5" t="n">
@@ -46140,7 +46140,7 @@
       </c>
       <c r="D701" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E701" s="5" t="n">
@@ -46268,7 +46268,7 @@
       </c>
       <c r="D703" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E703" s="5" t="n">
@@ -46333,7 +46333,7 @@
       </c>
       <c r="D704" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E704" s="5" t="n">
@@ -46399,7 +46399,7 @@
       </c>
       <c r="D705" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E705" s="5" t="n">
@@ -46528,7 +46528,7 @@
       </c>
       <c r="D707" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E707" s="5" t="n">
@@ -46719,7 +46719,7 @@
       </c>
       <c r="D710" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E710" s="5" t="n">
@@ -46845,7 +46845,7 @@
       </c>
       <c r="D712" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E712" s="5" t="n">
@@ -47036,7 +47036,7 @@
       </c>
       <c r="D715" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E715" s="5" t="n">
@@ -47357,7 +47357,7 @@
       </c>
       <c r="D720" s="5" t="inlineStr">
         <is>
-          <t>Bench</t>
+          <t>Flat bench</t>
         </is>
       </c>
       <c r="E720" s="5" t="n">
@@ -47487,7 +47487,7 @@
       </c>
       <c r="D722" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E722" s="5" t="n">
@@ -47552,7 +47552,7 @@
       </c>
       <c r="D723" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E723" s="5" t="n">
@@ -47618,7 +47618,7 @@
       </c>
       <c r="D724" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E724" s="5" t="n">
@@ -47810,7 +47810,7 @@
       </c>
       <c r="D727" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E727" s="5" t="n">
@@ -47875,7 +47875,7 @@
       </c>
       <c r="D728" s="5" t="inlineStr">
         <is>
-          <t>Kettlebell</t>
+          <t>Kettlebells</t>
         </is>
       </c>
       <c r="E728" s="5" t="n">
@@ -48007,7 +48007,7 @@
       </c>
       <c r="D730" s="5" t="inlineStr">
         <is>
-          <t>Bands, Mat</t>
+          <t>Mini bands, Mat</t>
         </is>
       </c>
       <c r="E730" s="5" t="n">
@@ -48070,7 +48070,7 @@
       </c>
       <c r="D731" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E731" s="5" t="n">
@@ -48133,7 +48133,7 @@
       </c>
       <c r="D732" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E732" s="5" t="n">
@@ -48196,7 +48196,7 @@
       </c>
       <c r="D733" s="5" t="inlineStr">
         <is>
-          <t>Cable</t>
+          <t>Cable station</t>
         </is>
       </c>
       <c r="E733" s="5" t="n">
@@ -48260,7 +48260,7 @@
       </c>
       <c r="D734" s="5" t="inlineStr">
         <is>
-          <t>Bands, Mat</t>
+          <t>Mini bands, Mat</t>
         </is>
       </c>
       <c r="E734" s="5" t="n">
@@ -48323,7 +48323,7 @@
       </c>
       <c r="D735" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E735" s="5" t="n">
@@ -48386,7 +48386,7 @@
       </c>
       <c r="D736" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E736" s="5" t="n">
@@ -48515,7 +48515,7 @@
       </c>
       <c r="D738" s="5" t="inlineStr">
         <is>
-          <t>Dumbbells, Bench</t>
+          <t>Dumbbells, Flat bench</t>
         </is>
       </c>
       <c r="E738" s="5" t="n">
@@ -48713,7 +48713,7 @@
       </c>
       <c r="D741" s="5" t="inlineStr">
         <is>
-          <t>Bands</t>
+          <t>Long resistance bands</t>
         </is>
       </c>
       <c r="E741" s="5" t="n">

</xml_diff>

<commit_message>
Phase 20 P2 (release and docs): honest Restore, hidden unset legal links, env:check values, production EAS env, no Face ID string, reviewer sheet test
- Restore purchases checks the entitlement afterwards: "No purchases to
  restore" when still free (en/es/pt-BR); Terms/Privacy hidden when unset
- env:check rejects non-https Terms/Privacy/Share URLs and personal
  mailboxes for support; eas.json production uses the production environment
- expo-secure-store faceIDPermission false (no NSFaceIDUsageDescription)
- reviewer sheet rebuilt (knee flags, BP, R8-06 notes) with a jest test that
  compares it to the seed
- launch-readiness: 44 h / 90 h, items 15 and 18 block the production build;
  the "checked by a certified coach" store line waits for the reviewer

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -3741,7 +3741,7 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>Shoulder, Recent surgery</t>
+          <t>Shoulder, Recent surgery, High blood pressure</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
@@ -11232,7 +11232,7 @@
       </c>
       <c r="I159" s="5" t="inlineStr">
         <is>
-          <t>Anchor the band high, kneel or stand, and pull your elbows down to your sides toward your back pockets.</t>
+          <t>Anchor the band high, sit or stand, and pull your elbows down to your sides toward your back pockets.</t>
         </is>
       </c>
       <c r="J159" s="5" t="inlineStr">
@@ -18755,7 +18755,7 @@
       </c>
       <c r="H274" s="5" t="inlineStr">
         <is>
-          <t>Hip, Shoulder, Pregnant / postpartum, Recent surgery, Knee</t>
+          <t>Hip, Shoulder, Pregnant / postpartum, Recent surgery, Knee, High blood pressure</t>
         </is>
       </c>
       <c r="I274" s="5" t="inlineStr">
@@ -20042,7 +20042,7 @@
       </c>
       <c r="H294" s="5" t="inlineStr">
         <is>
-          <t>Shoulder, Recent surgery, Knee</t>
+          <t>Shoulder, Recent surgery, Knee, High blood pressure</t>
         </is>
       </c>
       <c r="I294" s="5" t="inlineStr">
@@ -21601,7 +21601,7 @@
       </c>
       <c r="H318" s="5" t="inlineStr">
         <is>
-          <t>Lower back, Recent surgery</t>
+          <t>Lower back, Recent surgery, High blood pressure</t>
         </is>
       </c>
       <c r="I318" s="5" t="inlineStr">
@@ -31038,7 +31038,8 @@
       <c r="K463" s="5" t="inlineStr">
         <is>
           <t>Lower back: Bend forward (hold, no movement)
-Hip: Knee toward chest (hold, no movement)</t>
+Hip: Knee toward chest (hold, no movement)
+Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
       <c r="L463" s="5" t="inlineStr">
@@ -31478,7 +31479,7 @@
       </c>
       <c r="H470" s="5" t="inlineStr">
         <is>
-          <t>Recent surgery, Shoulder, Knee</t>
+          <t>Recent surgery, Shoulder, Knee, High blood pressure</t>
         </is>
       </c>
       <c r="I470" s="5" t="inlineStr">
@@ -31997,7 +31998,7 @@
       </c>
       <c r="H478" s="5" t="inlineStr">
         <is>
-          <t>Recent surgery, Pregnant / postpartum, Knee</t>
+          <t>Recent surgery, Pregnant / postpartum, Knee, High blood pressure</t>
         </is>
       </c>
       <c r="I478" s="5" t="inlineStr">
@@ -32063,7 +32064,8 @@
       </c>
       <c r="H479" s="5" t="inlineStr">
         <is>
-          <t>Recent surgery</t>
+          <t>Recent surgery
+REVIEWER: clinician decides whether this loads the knee / pivots the knee</t>
         </is>
       </c>
       <c r="I479" s="5" t="inlineStr">
@@ -32127,7 +32129,8 @@
       </c>
       <c r="H480" s="5" t="inlineStr">
         <is>
-          <t>Recent surgery</t>
+          <t>Recent surgery
+REVIEWER: clinician decides whether this loads the knee / pivots the knee</t>
         </is>
       </c>
       <c r="I480" s="5" t="inlineStr">
@@ -47465,7 +47468,8 @@
       <c r="K719" s="5" t="inlineStr">
         <is>
           <t>Lower back: Bend forward (full)
-Hip: Knee toward chest (full)</t>
+Hip: Knee toward chest (full)
+Knee: Bend the knee deep (partial)</t>
         </is>
       </c>
       <c r="L719" s="5" t="inlineStr">
@@ -48550,7 +48554,8 @@
       </c>
       <c r="H736" s="5" t="inlineStr">
         <is>
-          <t>Hip, Recent surgery</t>
+          <t>Hip, Recent surgery
+REVIEWER: clinician decides whether this loads the knee / pivots the knee</t>
         </is>
       </c>
       <c r="I736" s="5" t="inlineStr">
@@ -48613,7 +48618,8 @@
       </c>
       <c r="H737" s="5" t="inlineStr">
         <is>
-          <t>Hip, Recent surgery</t>
+          <t>Hip, Recent surgery
+REVIEWER: clinician decides whether this loads the knee / pivots the knee</t>
         </is>
       </c>
       <c r="I737" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Phase 23 (decision 3): the painful-joint budget counts only moves that move the joint
- movedAreas(): a joint tagged isometric (only holding still or
  stabilising) is not counted; used by the generator budget, the workout
  history (jointSets) and the test simulator.
- Seed tag cleanup where the joint only holds: wrist grip in dumbbell
  squats, RDLs, carries and shrugs; wrist on the floor in plank and bird
  dog; shoulder in the back squat and the suitcase carry; knee in reverse
  crunches; lower back in glute bridges and hip thrusts. seed.sql and the
  review sheet rebuilt.
- Tests per joint (knee, shoulder, lower back, hip, elbow/wrist, neck) with
  one moving and one isometric example: tags, history and generator; plus
  Daniel's knee list. They fail with the old rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -2911,7 +2911,7 @@
       <c r="K31" s="5" t="inlineStr">
         <is>
           <t>Shoulder: Carry weight (full)
-Wrist: Grip tight (full)
+Wrist: Grip tight (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
       </c>
@@ -3043,7 +3043,7 @@
         <is>
           <t>Shoulder: Arm overhead (partial)
 Hip: Leg behind you (partial)
-Wrist: Weight on your hands (partial)
+Wrist: Weight on your hands (hold, no movement)
 Knee: Kneel (full)
 Lower back: Arch your back (hold, no movement)</t>
         </is>
@@ -3497,7 +3497,7 @@
       <c r="K40" s="5" t="inlineStr">
         <is>
           <t>Shoulder: Push (hold, no movement)
-Wrist: Weight on your hands (partial)
+Wrist: Weight on your hands (hold, no movement)
 Lower back: Arch your back (hold, no movement)</t>
         </is>
       </c>
@@ -3692,7 +3692,7 @@
         <is>
           <t>Lower back: Bend forward (full)
 Hip: Knee toward chest (full)
-Knee: Bend the knee deep (partial)</t>
+Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
       <c r="L43" s="5" t="inlineStr">
@@ -3956,7 +3956,7 @@
           <t>Knee: Bend the knee deep (full)
 Hip: Deep squat (full)
 Ankle: Knee over toes (full)
-Wrist: Grip tight (full)</t>
+Wrist: Grip tight (hold, no movement)</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
@@ -4219,7 +4219,7 @@
       <c r="K51" s="5" t="inlineStr">
         <is>
           <t>Hip: Leg behind you (full)
-Lower back: Arch your back (partial)
+Lower back: Arch your back (hold, no movement)
 Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
@@ -4286,7 +4286,7 @@
         <is>
           <t>Hip: Knee toward chest (full)
 Lower back: Lift from the floor (full)
-Wrist: Grip tight (full)
+Wrist: Grip tight (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
       </c>
@@ -10845,7 +10845,7 @@
       <c r="K153" s="5" t="inlineStr">
         <is>
           <t>Shoulder: Carry weight (full)
-Wrist: Grip tight (partial)
+Wrist: Grip tight (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
       </c>
@@ -16156,7 +16156,7 @@
       <c r="K234" s="5" t="inlineStr">
         <is>
           <t>Shoulder: Carry weight (full)
-Wrist: Grip tight (full)
+Wrist: Grip tight (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
       </c>
@@ -16221,7 +16221,7 @@
       <c r="K235" s="5" t="inlineStr">
         <is>
           <t>Shoulder: Carry weight (full)
-Wrist: Grip tight (full)
+Wrist: Grip tight (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
       </c>
@@ -17728,7 +17728,7 @@
         <is>
           <t>Hip: Leg behind you (full)
 Hip: Stand on one leg (partial)
-Lower back: Arch your back (partial)
+Lower back: Arch your back (hold, no movement)
 Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
@@ -20696,7 +20696,7 @@
         <is>
           <t>Hip: Leg behind you (full)
 Hip: Leg out to the side (hold, no movement)
-Lower back: Arch your back (partial)
+Lower back: Arch your back (hold, no movement)
 Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
@@ -21221,7 +21221,7 @@
           <t>Knee: Bend the knee deep (full)
 Hip: Leg behind you (partial)
 Ankle: Knee over toes (partial)
-Wrist: Grip tight (full)</t>
+Wrist: Grip tight (hold, no movement)</t>
         </is>
       </c>
       <c r="L312" s="5" t="inlineStr">
@@ -21287,7 +21287,7 @@
           <t>Knee: Bend the knee deep (partial)
 Hip: Deep squat (partial)
 Ankle: Knee over toes (partial)
-Wrist: Grip tight (full)</t>
+Wrist: Grip tight (hold, no movement)</t>
         </is>
       </c>
       <c r="L313" s="5" t="inlineStr">
@@ -21352,7 +21352,7 @@
       <c r="K314" s="5" t="inlineStr">
         <is>
           <t>Hip: Leg behind you (full)
-Lower back: Arch your back (partial)
+Lower back: Arch your back (hold, no movement)
 Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
@@ -21420,7 +21420,7 @@
           <t>Knee: Bend the knee deep (full)
 Hip: Deep squat (full)
 Hip: Leg out to the side (partial)
-Wrist: Grip tight (full)</t>
+Wrist: Grip tight (hold, no movement)</t>
         </is>
       </c>
       <c r="L315" s="5" t="inlineStr">
@@ -21488,7 +21488,7 @@
           <t>Hip: Knee toward chest (full)
 Hip: Stand on one leg (full)
 Ankle: Balance and uneven ground (partial)
-Wrist: Grip tight (full)
+Wrist: Grip tight (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
       </c>
@@ -21616,8 +21616,8 @@
       </c>
       <c r="K318" s="5" t="inlineStr">
         <is>
-          <t>Shoulder: Carry weight (partial)
-Wrist: Grip tight (full)
+          <t>Shoulder: Carry weight (hold, no movement)
+Wrist: Grip tight (hold, no movement)
 Lower back: Lean to the side (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
@@ -21685,7 +21685,7 @@
         <is>
           <t>Hip: Knee toward chest (full)
 Shoulder: Raise arm in front (hold, no movement)
-Wrist: Grip tight (partial)
+Wrist: Grip tight (hold, no movement)
 Knee: Bend the knee deep (partial)</t>
         </is>
       </c>
@@ -22006,7 +22006,7 @@
 Hip: Deep squat (full)
 Ankle: Knee over toes (full)
 Lower back: Lift from the floor (hold, no movement)
-Shoulder: Turn arm outward (partial)</t>
+Shoulder: Turn arm outward (hold, no movement)</t>
         </is>
       </c>
       <c r="L324" s="5" t="inlineStr">
@@ -22071,7 +22071,7 @@
       <c r="K325" s="5" t="inlineStr">
         <is>
           <t>Hip: Leg behind you (full)
-Lower back: Arch your back (partial)
+Lower back: Arch your back (hold, no movement)
 Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
@@ -22138,7 +22138,7 @@
         <is>
           <t>Hip: Knee toward chest (full)
 Hip: Leg behind you (full)
-Wrist: Grip tight (full)
+Wrist: Grip tight (hold, no movement)
 Knee: Straighten with effort (hold, no movement)</t>
         </is>
       </c>
@@ -47469,7 +47469,7 @@
         <is>
           <t>Lower back: Bend forward (full)
 Hip: Knee toward chest (full)
-Knee: Bend the knee deep (partial)</t>
+Knee: Bend the knee deep (hold, no movement)</t>
         </is>
       </c>
       <c r="L719" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Phase 30: shoulder mobility & strength rehab program
- 13 draft rehab exercises (stretches, band, dumbbell, scapular) + stick
  equipment, i18n en/es/pt-BR, seed.sql and review sheet rebuilt
- Rehab category with the shoulder program: safety screen and affected-side
  question, sessions A/B/C, 6-week calendar, maintenance, "?" help, source
  credit, minor warning
- Player: 30 s holds / 30 s rest countdown, 10 s holds, side labels, block
  headers; load-raise suggestion after 2 easy, pain-free sessions (never in
  a week with pain); pain marks the exercise for review
- Local program store wired into family switch and account deletion
- security:check: track node-forge GHSA-86w9-cpqp-85rv (no fix released,
  CLI-only) as a warning; any other high/critical still fails
- Tests for program logic, screens and audit tracking; progress report

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YZKDqVTirwP3vm8p6KZMpS
</commit_message>
<xml_diff>
--- a/docs/review/exercise-review.xlsx
+++ b/docs/review/exercise-review.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Movements" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercises'!$A$1:$N$755</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exercises'!$A$1:$N$768</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B20" s="7">
-        <f>COUNTA(Exercises!$A$2:$A$755)</f>
+        <f>COUNTA(Exercises!$A$2:$A$768)</f>
         <v/>
       </c>
     </row>
@@ -781,7 +781,7 @@
         </is>
       </c>
       <c r="B21" s="7">
-        <f>COUNTIF(Exercises!$M$2:$M$755,"Approve")</f>
+        <f>COUNTIF(Exercises!$M$2:$M$768,"Approve")</f>
         <v/>
       </c>
     </row>
@@ -792,7 +792,7 @@
         </is>
       </c>
       <c r="B22" s="7">
-        <f>COUNTIF(Exercises!$M$2:$M$755,"Fix")</f>
+        <f>COUNTIF(Exercises!$M$2:$M$768,"Fix")</f>
         <v/>
       </c>
     </row>
@@ -856,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N755"/>
+  <dimension ref="A1:N768"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -49812,10 +49812,846 @@
       <c r="M755" s="6" t="n"/>
       <c r="N755" s="6" t="n"/>
     </row>
+    <row r="756">
+      <c r="A756" s="5" t="inlineStr">
+        <is>
+          <t>pendulum_swing</t>
+        </is>
+      </c>
+      <c r="B756" s="5" t="inlineStr">
+        <is>
+          <t>Pendulum swing</t>
+        </is>
+      </c>
+      <c r="C756" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.7
+Front shoulders (Deltoid · front head): secondary, 0.5</t>
+        </is>
+      </c>
+      <c r="D756" s="5" t="inlineStr">
+        <is>
+          <t>Bodyweight</t>
+        </is>
+      </c>
+      <c r="E756" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F756" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G756" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support</t>
+        </is>
+      </c>
+      <c r="H756" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I756" s="5" t="inlineStr">
+        <is>
+          <t>Lean forward with one hand on a table and let the other arm hang loose. Move your body so the arm swings gently forward and back, then side to side, then in small circles; switch arms. Keep your back straight and knees slightly bent.</t>
+        </is>
+      </c>
+      <c r="J756" s="5" t="inlineStr">
+        <is>
+          <t>Main work, Warm-up: mobility · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K756" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Raise arm in front (partial)
+Shoulder: Raise arm to the side (partial)</t>
+        </is>
+      </c>
+      <c r="L756" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M756" s="6" t="n"/>
+      <c r="N756" s="6" t="n"/>
+    </row>
+    <row r="757">
+      <c r="A757" s="5" t="inlineStr">
+        <is>
+          <t>crossover_arm_stretch</t>
+        </is>
+      </c>
+      <c r="B757" s="5" t="inlineStr">
+        <is>
+          <t>Crossover arm stretch</t>
+        </is>
+      </c>
+      <c r="C757" s="5" t="inlineStr">
+        <is>
+          <t>Rear shoulders (Deltoid · rear head): primary, 0.8
+Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): secondary, 0.4</t>
+        </is>
+      </c>
+      <c r="D757" s="5" t="inlineStr">
+        <is>
+          <t>Bodyweight</t>
+        </is>
+      </c>
+      <c r="E757" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F757" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G757" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support, Seated</t>
+        </is>
+      </c>
+      <c r="H757" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I757" s="5" t="inlineStr">
+        <is>
+          <t>Relax your shoulders. With the other hand on your arm, just above the elbow, bring the arm across your chest until you feel the stretch at the back of the shoulder. Hold 30 s, release 30 s. Don't pull on the elbow itself.</t>
+        </is>
+      </c>
+      <c r="J757" s="5" t="inlineStr">
+        <is>
+          <t>Main work, Cool-down: stretch · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K757" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Raise arm in front (partial)</t>
+        </is>
+      </c>
+      <c r="L757" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Raise arm in front</t>
+        </is>
+      </c>
+      <c r="M757" s="6" t="n"/>
+      <c r="N757" s="6" t="n"/>
+    </row>
+    <row r="758">
+      <c r="A758" s="5" t="inlineStr">
+        <is>
+          <t>stick_internal_rotation_stretch</t>
+        </is>
+      </c>
+      <c r="B758" s="5" t="inlineStr">
+        <is>
+          <t>Stick internal rotation stretch</t>
+        </is>
+      </c>
+      <c r="C758" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Front shoulders (Deltoid · front head): secondary, 0.4</t>
+        </is>
+      </c>
+      <c r="D758" s="5" t="inlineStr">
+        <is>
+          <t>Light stick (broom handle)</t>
+        </is>
+      </c>
+      <c r="E758" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F758" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G758" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support</t>
+        </is>
+      </c>
+      <c r="H758" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I758" s="5" t="inlineStr">
+        <is>
+          <t>Hold a light stick behind your back at hip height with both hands. With the hand on your good side, pull the stick to the side until you feel a gentle, painless pull in the affected shoulder. Hold 30 s, release 30 s. Don't lean or twist your body.</t>
+        </is>
+      </c>
+      <c r="J758" s="5" t="inlineStr">
+        <is>
+          <t>Main work, Cool-down: stretch · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K758" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward (partial)
+Shoulder: Reach behind your back (partial)</t>
+        </is>
+      </c>
+      <c r="L758" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward</t>
+        </is>
+      </c>
+      <c r="M758" s="6" t="n"/>
+      <c r="N758" s="6" t="n"/>
+    </row>
+    <row r="759">
+      <c r="A759" s="5" t="inlineStr">
+        <is>
+          <t>stick_external_rotation_stretch</t>
+        </is>
+      </c>
+      <c r="B759" s="5" t="inlineStr">
+        <is>
+          <t>Stick external rotation stretch</t>
+        </is>
+      </c>
+      <c r="C759" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Rear shoulders (Deltoid · rear head): secondary, 0.3</t>
+        </is>
+      </c>
+      <c r="D759" s="5" t="inlineStr">
+        <is>
+          <t>Light stick (broom handle)</t>
+        </is>
+      </c>
+      <c r="E759" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F759" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G759" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support, Seated</t>
+        </is>
+      </c>
+      <c r="H759" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I759" s="5" t="inlineStr">
+        <is>
+          <t>Keep the elbow of the affected side against your body, bent to 90°. Hold one end of a light stick with that hand and the other end with your good hand. Push the stick toward the affected side, turning the forearm out, until you feel a gentle, painless pull. Hold 30 s, release 30 s. Keep your hips facing forward.</t>
+        </is>
+      </c>
+      <c r="J759" s="5" t="inlineStr">
+        <is>
+          <t>Main work, Cool-down: stretch · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K759" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm outward (partial)</t>
+        </is>
+      </c>
+      <c r="L759" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm outward</t>
+        </is>
+      </c>
+      <c r="M759" s="6" t="n"/>
+      <c r="N759" s="6" t="n"/>
+    </row>
+    <row r="760">
+      <c r="A760" s="5" t="inlineStr">
+        <is>
+          <t>sleeper_stretch</t>
+        </is>
+      </c>
+      <c r="B760" s="5" t="inlineStr">
+        <is>
+          <t>Sleeper stretch</t>
+        </is>
+      </c>
+      <c r="C760" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Rear shoulders (Deltoid · rear head): secondary, 0.5</t>
+        </is>
+      </c>
+      <c r="D760" s="5" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="E760" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F760" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G760" s="5" t="inlineStr">
+        <is>
+          <t>With support, Standing</t>
+        </is>
+      </c>
+      <c r="H760" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I760" s="5" t="inlineStr">
+        <is>
+          <t>Lie on the affected side with a pillow under your head. Put the bottom arm in front of you, elbow bent to 90° and hand pointing up. With the other hand, slowly push the forearm down toward the floor until you feel the stretch at the back of the shoulder. Hold 30 s, release 30 s. Push on the forearm, never the wrist, and don't bend the wrist.</t>
+        </is>
+      </c>
+      <c r="J760" s="5" t="inlineStr">
+        <is>
+          <t>Main work, Cool-down: stretch · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K760" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward (partial)</t>
+        </is>
+      </c>
+      <c r="L760" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward</t>
+        </is>
+      </c>
+      <c r="M760" s="6" t="n"/>
+      <c r="N760" s="6" t="n"/>
+    </row>
+    <row r="761">
+      <c r="A761" s="5" t="inlineStr">
+        <is>
+          <t>band_external_rotation_90</t>
+        </is>
+      </c>
+      <c r="B761" s="5" t="inlineStr">
+        <is>
+          <t>Band external rotation with the arm at 90°</t>
+        </is>
+      </c>
+      <c r="C761" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Rear shoulders (Deltoid · rear head): secondary, 0.4</t>
+        </is>
+      </c>
+      <c r="D761" s="5" t="inlineStr">
+        <is>
+          <t>Long resistance bands</t>
+        </is>
+      </c>
+      <c r="E761" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F761" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G761" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support</t>
+        </is>
+      </c>
+      <c r="H761" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I761" s="5" t="inlineStr">
+        <is>
+          <t>Anchor the band in front of you. Lift the arm out to shoulder height, elbow bent to 90° and hand pointing forward. Turn the hand up until it's in line with your head, without dropping the elbow; return slowly. Keep the elbow level with the shoulder.</t>
+        </is>
+      </c>
+      <c r="J761" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K761" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm outward (partial)
+Shoulder: Raise arm to the side (hold, no movement)
+Wrist: Grip tight (hold, no movement)</t>
+        </is>
+      </c>
+      <c r="L761" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm outward</t>
+        </is>
+      </c>
+      <c r="M761" s="6" t="n"/>
+      <c r="N761" s="6" t="n"/>
+    </row>
+    <row r="762">
+      <c r="A762" s="5" t="inlineStr">
+        <is>
+          <t>band_internal_rotation</t>
+        </is>
+      </c>
+      <c r="B762" s="5" t="inlineStr">
+        <is>
+          <t>Band internal rotation, elbow at your side</t>
+        </is>
+      </c>
+      <c r="C762" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Chest (Pectoralis major): secondary, 0.3</t>
+        </is>
+      </c>
+      <c r="D762" s="5" t="inlineStr">
+        <is>
+          <t>Long resistance bands</t>
+        </is>
+      </c>
+      <c r="E762" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F762" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G762" s="5" t="inlineStr">
+        <is>
+          <t>Standing, With support, Seated</t>
+        </is>
+      </c>
+      <c r="H762" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I762" s="5" t="inlineStr">
+        <is>
+          <t>Anchor the band at your side, at elbow height. Keep the elbow against your body, bent to 90°. Bring the hand in across the front of your belly; return slowly. Keep pressing the elbow into your side.</t>
+        </is>
+      </c>
+      <c r="J762" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K762" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward (partial)
+Wrist: Grip tight (partial)</t>
+        </is>
+      </c>
+      <c r="L762" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward</t>
+        </is>
+      </c>
+      <c r="M762" s="6" t="n"/>
+      <c r="N762" s="6" t="n"/>
+    </row>
+    <row r="763">
+      <c r="A763" s="5" t="inlineStr">
+        <is>
+          <t>kneeling_thumbs_up_raise</t>
+        </is>
+      </c>
+      <c r="B763" s="5" t="inlineStr">
+        <is>
+          <t>Thumbs-up side raise on a bench</t>
+        </is>
+      </c>
+      <c r="C763" s="5" t="inlineStr">
+        <is>
+          <t>Front shoulders (Deltoid · front head): primary, 0.7
+Rear shoulders (Deltoid · rear head): primary, 0.6
+Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): secondary, 0.5
+Traps (Trapezius): secondary, 0.4</t>
+        </is>
+      </c>
+      <c r="D763" s="5" t="inlineStr">
+        <is>
+          <t>Dumbbells</t>
+        </is>
+      </c>
+      <c r="E763" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F763" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G763" s="5" t="inlineStr">
+        <is>
+          <t>With support, Standing</t>
+        </is>
+      </c>
+      <c r="H763" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I763" s="5" t="inlineStr">
+        <is>
+          <t>One knee and one hand on a bench or chair, back flat. Let the other arm hang holding a light dumbbell. Raise the arm out to the side to shoulder height, turning the hand until the thumb points up; lower over 5 counts. Pick a weight that makes the last reps hard but never painful.</t>
+        </is>
+      </c>
+      <c r="J763" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K763" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Raise arm to the side (partial)
+Wrist: Grip tight (partial)</t>
+        </is>
+      </c>
+      <c r="L763" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Raise arm to the side</t>
+        </is>
+      </c>
+      <c r="M763" s="6" t="n"/>
+      <c r="N763" s="6" t="n"/>
+    </row>
+    <row r="764">
+      <c r="A764" s="5" t="inlineStr">
+        <is>
+          <t>prone_scapula_setting</t>
+        </is>
+      </c>
+      <c r="B764" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder blade setting, face down</t>
+        </is>
+      </c>
+      <c r="C764" s="5" t="inlineStr">
+        <is>
+          <t>Upper back (Rhomboids and middle trapezius): primary, 0.7
+Traps (Trapezius): secondary, 0.5</t>
+        </is>
+      </c>
+      <c r="D764" s="5" t="inlineStr">
+        <is>
+          <t>Mat</t>
+        </is>
+      </c>
+      <c r="E764" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F764" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G764" s="5" t="inlineStr">
+        <is>
+          <t>With support, Standing</t>
+        </is>
+      </c>
+      <c r="H764" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I764" s="5" t="inlineStr">
+        <is>
+          <t>Lie face down with your arms by your sides (a pillow under the forehead if needed). Draw your shoulder blades together and down, ease off halfway and hold 10 s; relax and repeat. Keep your neck relaxed.</t>
+        </is>
+      </c>
+      <c r="J764" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K764" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Pull (hold, no movement)</t>
+        </is>
+      </c>
+      <c r="L764" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M764" s="6" t="n"/>
+      <c r="N764" s="6" t="n"/>
+    </row>
+    <row r="765">
+      <c r="A765" s="5" t="inlineStr">
+        <is>
+          <t>prone_table_scapular_retraction</t>
+        </is>
+      </c>
+      <c r="B765" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder blade squeeze, face down on a bed</t>
+        </is>
+      </c>
+      <c r="C765" s="5" t="inlineStr">
+        <is>
+          <t>Upper back (Rhomboids and middle trapezius): primary, 0.8
+Traps (Trapezius): secondary, 0.5</t>
+        </is>
+      </c>
+      <c r="D765" s="5" t="inlineStr">
+        <is>
+          <t>Dumbbells</t>
+        </is>
+      </c>
+      <c r="E765" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F765" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G765" s="5" t="inlineStr">
+        <is>
+          <t>With support, Standing</t>
+        </is>
+      </c>
+      <c r="H765" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I765" s="5" t="inlineStr">
+        <is>
+          <t>Lie face down on a firm bed or table with the affected arm hanging off the edge, elbow straight. Lift the weight only by squeezing the shoulder blade toward your spine; lower slowly. Don't shrug toward your ear.</t>
+        </is>
+      </c>
+      <c r="J765" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K765" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Pull (partial)
+Wrist: Grip tight (partial)</t>
+        </is>
+      </c>
+      <c r="L765" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Pull</t>
+        </is>
+      </c>
+      <c r="M765" s="6" t="n"/>
+      <c r="N765" s="6" t="n"/>
+    </row>
+    <row r="766">
+      <c r="A766" s="5" t="inlineStr">
+        <is>
+          <t>prone_horizontal_abduction</t>
+        </is>
+      </c>
+      <c r="B766" s="5" t="inlineStr">
+        <is>
+          <t>Face-down side arm raise</t>
+        </is>
+      </c>
+      <c r="C766" s="5" t="inlineStr">
+        <is>
+          <t>Rear shoulders (Deltoid · rear head): primary, 0.8
+Upper back (Rhomboids and middle trapezius): primary, 0.6
+Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): secondary, 0.4</t>
+        </is>
+      </c>
+      <c r="D766" s="5" t="inlineStr">
+        <is>
+          <t>Dumbbells</t>
+        </is>
+      </c>
+      <c r="E766" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F766" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G766" s="5" t="inlineStr">
+        <is>
+          <t>With support, Standing</t>
+        </is>
+      </c>
+      <c r="H766" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I766" s="5" t="inlineStr">
+        <is>
+          <t>Lie face down on a bed or table with the affected arm hanging down. With the arm straight, raise it out to the side to eye level; lower slowly and under control.</t>
+        </is>
+      </c>
+      <c r="J766" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K766" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Raise arm to the side (partial)
+Wrist: Grip tight (partial)</t>
+        </is>
+      </c>
+      <c r="L766" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Raise arm to the side</t>
+        </is>
+      </c>
+      <c r="M766" s="6" t="n"/>
+      <c r="N766" s="6" t="n"/>
+    </row>
+    <row r="767">
+      <c r="A767" s="5" t="inlineStr">
+        <is>
+          <t>supine_shoulder_rotation_90</t>
+        </is>
+      </c>
+      <c r="B767" s="5" t="inlineStr">
+        <is>
+          <t>Lying shoulder rotation at 90°</t>
+        </is>
+      </c>
+      <c r="C767" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Rear shoulders (Deltoid · rear head): secondary, 0.3
+Chest (Pectoralis major): secondary, 0.2</t>
+        </is>
+      </c>
+      <c r="D767" s="5" t="inlineStr">
+        <is>
+          <t>Dumbbells, Mat</t>
+        </is>
+      </c>
+      <c r="E767" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F767" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G767" s="5" t="inlineStr">
+        <is>
+          <t>With support, Standing</t>
+        </is>
+      </c>
+      <c r="H767" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I767" s="5" t="inlineStr">
+        <is>
+          <t>Lie on your back with the arm out at shoulder height, elbow bent to 90° and fingers pointing up. Keeping the elbow on the floor, turn the forearm forward and back in an arc. If 90° hurts, lower the elbow to 45°. Pick a weight that makes the last reps hard but never painful.</t>
+        </is>
+      </c>
+      <c r="J767" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K767" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm outward (partial)
+Shoulder: Turn arm inward (partial)
+Shoulder: Raise arm to the side (hold, no movement)
+Wrist: Grip tight (partial)</t>
+        </is>
+      </c>
+      <c r="L767" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm outward
+Shoulder: Turn arm inward</t>
+        </is>
+      </c>
+      <c r="M767" s="6" t="n"/>
+      <c r="N767" s="6" t="n"/>
+    </row>
+    <row r="768">
+      <c r="A768" s="5" t="inlineStr">
+        <is>
+          <t>side_lying_internal_rotation</t>
+        </is>
+      </c>
+      <c r="B768" s="5" t="inlineStr">
+        <is>
+          <t>Side-lying internal rotation</t>
+        </is>
+      </c>
+      <c r="C768" s="5" t="inlineStr">
+        <is>
+          <t>Rotator cuff (Supraspinatus, infraspinatus, teres minor, subscapularis): primary, 0.8
+Chest (Pectoralis major): secondary, 0.2</t>
+        </is>
+      </c>
+      <c r="D768" s="5" t="inlineStr">
+        <is>
+          <t>Dumbbells, Mat</t>
+        </is>
+      </c>
+      <c r="E768" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F768" s="5" t="inlineStr">
+        <is>
+          <t>13+ (teens)</t>
+        </is>
+      </c>
+      <c r="G768" s="5" t="inlineStr">
+        <is>
+          <t>With support, Standing</t>
+        </is>
+      </c>
+      <c r="H768" s="5" t="inlineStr">
+        <is>
+          <t>Recent surgery</t>
+        </is>
+      </c>
+      <c r="I768" s="5" t="inlineStr">
+        <is>
+          <t>Lie on the affected side with a pillow or folded towel under your head. Keep the bottom elbow by your side, bent to 90°. Turn the forearm up toward your belly until it's vertical; lower slowly. Don't let your body roll back.</t>
+        </is>
+      </c>
+      <c r="J768" s="5" t="inlineStr">
+        <is>
+          <t>Main work · recovery plan only</t>
+        </is>
+      </c>
+      <c r="K768" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward (partial)
+Wrist: Grip tight (partial)</t>
+        </is>
+      </c>
+      <c r="L768" s="5" t="inlineStr">
+        <is>
+          <t>Shoulder: Turn arm inward</t>
+        </is>
+      </c>
+      <c r="M768" s="6" t="n"/>
+      <c r="N768" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N755"/>
+  <autoFilter ref="A1:N768"/>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M755" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Approve or Fix." prompt="Approve, or Fix and explain in Comment." type="list">
+    <dataValidation sqref="M2:M768" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choose Approve or Fix." prompt="Approve, or Fix and explain in Comment." type="list">
       <formula1>"Approve,Fix"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>